<commit_message>
docs: replace 400-hour build guess with bottom-up estimate
The side-business plan assumed ~400 hours to build the product, carried
over from the full-time calendar rather than estimated per task. A
bottom-up estimate with AI-assisted coding and the borrowed open-source
components puts demo-ready at ~60-120 hours and pilot-ready at ~100-190.

- 06: add an itemized build-estimate table; re-time Phase 0 to weeks 1-4
  and Phase 1 to weeks 5-8, with weeks 9-13 for pilot support
- README and 05: re-time the 90-day plans to match
- 08 and the side-business model: 150 build hours, sales one quarter
  earlier; Base case now ~$15k at risk, profitable from month 7, and
  ~$199k / ~$361k pre-tax profit in years 2-3 at ~22-27 hours a week

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01TDEQCSX5jr3s79EPtgeMEg
</commit_message>
<xml_diff>
--- a/docs/business/financial-model-side-business.xlsx
+++ b/docs/business/financial-model-side-business.xlsx
@@ -605,7 +605,7 @@
     <t xml:space="preserve">Sales Plan: new clients signed per quarter</t>
   </si>
   <si>
-    <t xml:space="preserve">Side business: new signed clients per quarter. Q1 = Oct-Dec 2026. Part-time build means the first client lands around month 7-9.</t>
+    <t xml:space="preserve">Side business: new signed clients per quarter. Q1 = Oct-Dec 2026. The product takes ~100-190 hours to pilot-ready (~6-12 weeks part-time), so the first client lands around month 4-6.</t>
   </si>
   <si>
     <t xml:space="preserve">Scenario</t>
@@ -656,7 +656,7 @@
     <t xml:space="preserve">Conservative</t>
   </si>
   <si>
-    <t xml:space="preserve">Side-business Base: product built part-time (~20 h/week) through ~month 6; one design partner in Q3 and one in Q4. Then roughly one new client per quarter in Year 2 and 1-2 per quarter in Year 3, from warm intros and 1-2 MSP partners. No Enterprise tier: its support load doesn't fit around a day job. Conservative is roughly half; Upside assumes an MSP partner feeds deals.</t>
+    <t xml:space="preserve">Side-business Base: product built part-time (~15-20 h/week) in ~8-10 weeks; first design partner in Q2, then roughly one new client per quarter plus a Firm-tier client every other quarter, from warm intros and 1-2 MSP partners. No Enterprise tier: its support load doesn't fit around a day job. Conservative is slower; Upside assumes an MSP partner feeds deals. Sales capacity, not the build, is the bottleneck.</t>
   </si>
   <si>
     <t xml:space="preserve">Base</t>
@@ -1944,11 +1944,11 @@
       </c>
       <c r="B5" s="9" t="n">
         <f aca="false">SUMIF(Projection!$B$3:$AK$3,1,Projection!$B$7:$AK$7)+SUMIF(Projection!$B$3:$AK$3,1,Projection!$B$8:$AK$8)+SUMIF(Projection!$B$3:$AK$3,1,Projection!$B$9:$AK$9)</f>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C5" s="9" t="n">
         <f aca="false">SUMIF(Projection!$B$3:$AK$3,2,Projection!$B$7:$AK$7)+SUMIF(Projection!$B$3:$AK$3,2,Projection!$B$8:$AK$8)+SUMIF(Projection!$B$3:$AK$3,2,Projection!$B$9:$AK$9)</f>
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D5" s="9" t="n">
         <f aca="false">SUMIF(Projection!$B$3:$AK$3,3,Projection!$B$7:$AK$7)+SUMIF(Projection!$B$3:$AK$3,3,Projection!$B$8:$AK$8)+SUMIF(Projection!$B$3:$AK$3,3,Projection!$B$9:$AK$9)</f>
@@ -1964,15 +1964,15 @@
       </c>
       <c r="B6" s="9" t="n">
         <f aca="false">INDEX(Projection!$B$15:$AK$15,1,12*1)</f>
-        <v>1.95679805531781</v>
+        <v>2.89721249784328</v>
       </c>
       <c r="C6" s="9" t="n">
         <f aca="false">INDEX(Projection!$B$15:$AK$15,1,12*2)</f>
-        <v>7.50599624133305</v>
+        <v>9.29343618164458</v>
       </c>
       <c r="D6" s="9" t="n">
         <f aca="false">INDEX(Projection!$B$15:$AK$15,1,12*3)</f>
-        <v>13.4413415507854</v>
+        <v>15.0744847493789</v>
       </c>
       <c r="E6" s="2"/>
     </row>
@@ -1987,11 +1987,11 @@
       </c>
       <c r="B8" s="11" t="n">
         <f aca="false">SUMIF(Projection!$B$3:$AK$3,1,Projection!$B$18:$AK$18)</f>
-        <v>32001.05</v>
+        <v>38324.9</v>
       </c>
       <c r="C8" s="11" t="n">
         <f aca="false">SUMIF(Projection!$B$3:$AK$3,2,Projection!$B$18:$AK$18)</f>
-        <v>76649.8</v>
+        <v>102327</v>
       </c>
       <c r="D8" s="11" t="n">
         <f aca="false">SUMIF(Projection!$B$3:$AK$3,3,Projection!$B$18:$AK$18)</f>
@@ -2007,11 +2007,11 @@
       </c>
       <c r="B9" s="11" t="n">
         <f aca="false">SUMIF(Projection!$B$3:$AK$3,1,Projection!$B$19:$AK$19)</f>
-        <v>16500</v>
+        <v>21000</v>
       </c>
       <c r="C9" s="11" t="n">
         <f aca="false">SUMIF(Projection!$B$3:$AK$3,2,Projection!$B$19:$AK$19)</f>
-        <v>42000</v>
+        <v>54000</v>
       </c>
       <c r="D9" s="11" t="n">
         <f aca="false">SUMIF(Projection!$B$3:$AK$3,3,Projection!$B$19:$AK$19)</f>
@@ -2025,15 +2025,15 @@
       </c>
       <c r="B10" s="11" t="n">
         <f aca="false">SUMIF(Projection!$B$3:$AK$3,1,Projection!$B$20:$AK$20)</f>
-        <v>7659.63853359694</v>
+        <v>17129.8859739423</v>
       </c>
       <c r="C10" s="11" t="n">
         <f aca="false">SUMIF(Projection!$B$3:$AK$3,2,Projection!$B$20:$AK$20)</f>
-        <v>138142.7707536</v>
+        <v>184138.978378741</v>
       </c>
       <c r="D10" s="11" t="n">
         <f aca="false">SUMIF(Projection!$B$3:$AK$3,3,Projection!$B$20:$AK$20)</f>
-        <v>315212.989093533</v>
+        <v>360547.960791181</v>
       </c>
       <c r="E10" s="2" t="s">
         <v>35</v>
@@ -2045,15 +2045,15 @@
       </c>
       <c r="B11" s="12" t="n">
         <f aca="false">SUM(B8:B10)</f>
-        <v>56160.6885335969</v>
+        <v>76454.7859739423</v>
       </c>
       <c r="C11" s="12" t="n">
         <f aca="false">SUM(C8:C10)</f>
-        <v>256792.5707536</v>
+        <v>340465.978378741</v>
       </c>
       <c r="D11" s="12" t="n">
         <f aca="false">SUM(D8:D10)</f>
-        <v>471539.989093533</v>
+        <v>516874.960791181</v>
       </c>
       <c r="E11" s="2"/>
     </row>
@@ -2063,15 +2063,15 @@
       </c>
       <c r="B12" s="12" t="n">
         <f aca="false">SUMIF(Projection!$B$3:$AK$3,1,Projection!$B$28:$AK$28)</f>
-        <v>26589.3249643787</v>
+        <v>40450.4779557818</v>
       </c>
       <c r="C12" s="12" t="n">
         <f aca="false">SUMIF(Projection!$B$3:$AK$3,2,Projection!$B$28:$AK$28)</f>
-        <v>182835.338382553</v>
+        <v>241993.889786455</v>
       </c>
       <c r="D12" s="12" t="n">
         <f aca="false">SUMIF(Projection!$B$3:$AK$3,3,Projection!$B$28:$AK$28)</f>
-        <v>369401.190620999</v>
+        <v>413479.532098658</v>
       </c>
       <c r="E12" s="2"/>
     </row>
@@ -2081,15 +2081,15 @@
       </c>
       <c r="B13" s="13" t="n">
         <f aca="false">IF(B11=0,0,B12/B11)</f>
-        <v>0.473450836495216</v>
+        <v>0.52907711977074</v>
       </c>
       <c r="C13" s="13" t="n">
         <f aca="false">IF(C11=0,0,C12/C11)</f>
-        <v>0.71199621486709</v>
+        <v>0.710772603297404</v>
       </c>
       <c r="D13" s="13" t="n">
         <f aca="false">IF(D11=0,0,D12/D11)</f>
-        <v>0.783393135608964</v>
+        <v>0.79996046135751</v>
       </c>
       <c r="E13" s="2"/>
     </row>
@@ -2117,15 +2117,15 @@
       </c>
       <c r="B15" s="12" t="n">
         <f aca="false">B12-B14</f>
-        <v>-5310.67503562126</v>
+        <v>8550.47795578176</v>
       </c>
       <c r="C15" s="12" t="n">
         <f aca="false">C12-C14</f>
-        <v>139935.338382553</v>
+        <v>199093.889786455</v>
       </c>
       <c r="D15" s="12" t="n">
         <f aca="false">D12-D14</f>
-        <v>316601.190620999</v>
+        <v>360679.532098658</v>
       </c>
       <c r="E15" s="2"/>
     </row>
@@ -2153,15 +2153,15 @@
       </c>
       <c r="B17" s="12" t="n">
         <f aca="false">INDEX(Projection!$B$45:$AK$45,1,12*1)</f>
-        <v>-10810.6750356213</v>
+        <v>3050.47795578176</v>
       </c>
       <c r="C17" s="12" t="n">
         <f aca="false">INDEX(Projection!$B$45:$AK$45,1,12*2)</f>
-        <v>129124.663346932</v>
+        <v>202144.367742237</v>
       </c>
       <c r="D17" s="12" t="n">
         <f aca="false">INDEX(Projection!$B$45:$AK$45,1,12*3)</f>
-        <v>445725.853967931</v>
+        <v>562823.899840895</v>
       </c>
       <c r="E17" s="2" t="s">
         <v>43</v>
@@ -2173,15 +2173,15 @@
       </c>
       <c r="B18" s="12" t="n">
         <f aca="false">INDEX(Projection!$B$47:$AK$47,1,12*1)</f>
-        <v>64960.8808247006</v>
+        <v>81115.2507917335</v>
       </c>
       <c r="C18" s="12" t="n">
         <f aca="false">INDEX(Projection!$B$47:$AK$47,1,12*2)</f>
-        <v>219823.545694821</v>
+        <v>279533.691883004</v>
       </c>
       <c r="D18" s="12" t="n">
         <f aca="false">INDEX(Projection!$B$47:$AK$47,1,12*3)</f>
-        <v>404371.157295782</v>
+        <v>459283.756976181</v>
       </c>
       <c r="E18" s="2" t="s">
         <v>45</v>
@@ -2218,7 +2218,7 @@
       </c>
       <c r="B21" s="15" t="n">
         <f aca="false">IF(MIN(Projection!$B$48:$AK$48)=999,"Not within 36 months",MIN(Projection!$B$48:$AK$48))</f>
-        <v>10</v>
+        <v>7</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2227,7 +2227,7 @@
       </c>
       <c r="B22" s="12" t="n">
         <f aca="false">MIN(Projection!$B$45:$AK$45)</f>
-        <v>-23108.2910065466</v>
+        <v>-15133.2910065466</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2236,7 +2236,7 @@
       </c>
       <c r="B23" s="16" t="n">
         <f aca="false">MAX(0,-B22)</f>
-        <v>23108.2910065466</v>
+        <v>15133.2910065466</v>
       </c>
       <c r="E23" s="2" t="s">
         <v>52</v>
@@ -2248,7 +2248,7 @@
       </c>
       <c r="B24" s="9" t="n">
         <f aca="false">Projection!$AK$15</f>
-        <v>13.4413415507854</v>
+        <v>15.0744847493789</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3354,28 +3354,28 @@
         <v>0</v>
       </c>
       <c r="E5" s="23" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F5" s="23" t="n">
+        <v>0</v>
+      </c>
+      <c r="G5" s="23" t="n">
         <v>1</v>
       </c>
-      <c r="G5" s="23" t="n">
-        <v>0</v>
-      </c>
       <c r="H5" s="23" t="n">
+        <v>0</v>
+      </c>
+      <c r="I5" s="23" t="n">
         <v>1</v>
-      </c>
-      <c r="I5" s="23" t="n">
-        <v>0</v>
       </c>
       <c r="J5" s="23" t="n">
         <v>1</v>
       </c>
       <c r="K5" s="23" t="n">
+        <v>0</v>
+      </c>
+      <c r="L5" s="23" t="n">
         <v>1</v>
-      </c>
-      <c r="L5" s="23" t="n">
-        <v>0</v>
       </c>
       <c r="M5" s="23" t="n">
         <v>1</v>
@@ -3385,7 +3385,7 @@
       </c>
       <c r="O5" s="15" t="n">
         <f aca="false">SUM(C5:N5)</f>
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="P5" s="29" t="s">
         <v>182</v>
@@ -3408,35 +3408,35 @@
         <v>0</v>
       </c>
       <c r="F6" s="23" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G6" s="23" t="n">
+        <v>0</v>
+      </c>
+      <c r="H6" s="23" t="n">
+        <v>0</v>
+      </c>
+      <c r="I6" s="23" t="n">
         <v>1</v>
       </c>
-      <c r="H6" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="I6" s="23" t="n">
-        <v>0</v>
-      </c>
       <c r="J6" s="23" t="n">
+        <v>0</v>
+      </c>
+      <c r="K6" s="23" t="n">
         <v>1</v>
       </c>
-      <c r="K6" s="23" t="n">
-        <v>0</v>
-      </c>
       <c r="L6" s="23" t="n">
+        <v>0</v>
+      </c>
+      <c r="M6" s="23" t="n">
         <v>1</v>
-      </c>
-      <c r="M6" s="23" t="n">
-        <v>0</v>
       </c>
       <c r="N6" s="23" t="n">
         <v>1</v>
       </c>
       <c r="O6" s="15" t="n">
         <f aca="false">SUM(C6:N6)</f>
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="P6" s="29"/>
     </row>
@@ -3500,13 +3500,13 @@
         <v>0</v>
       </c>
       <c r="D8" s="23" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E8" s="23" t="n">
+        <v>0</v>
+      </c>
+      <c r="F8" s="23" t="n">
         <v>1</v>
-      </c>
-      <c r="F8" s="23" t="n">
-        <v>0</v>
       </c>
       <c r="G8" s="23" t="n">
         <v>1</v>
@@ -3534,7 +3534,7 @@
       </c>
       <c r="O8" s="15" t="n">
         <f aca="false">SUM(C8:N8)</f>
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="P8" s="29"/>
     </row>
@@ -3552,28 +3552,28 @@
         <v>0</v>
       </c>
       <c r="E9" s="23" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F9" s="23" t="n">
+        <v>0</v>
+      </c>
+      <c r="G9" s="23" t="n">
         <v>1</v>
       </c>
-      <c r="G9" s="23" t="n">
-        <v>0</v>
-      </c>
       <c r="H9" s="23" t="n">
+        <v>0</v>
+      </c>
+      <c r="I9" s="23" t="n">
         <v>1</v>
-      </c>
-      <c r="I9" s="23" t="n">
-        <v>0</v>
       </c>
       <c r="J9" s="23" t="n">
         <v>1</v>
       </c>
       <c r="K9" s="23" t="n">
+        <v>0</v>
+      </c>
+      <c r="L9" s="23" t="n">
         <v>1</v>
-      </c>
-      <c r="L9" s="23" t="n">
-        <v>0</v>
       </c>
       <c r="M9" s="23" t="n">
         <v>1</v>
@@ -3583,7 +3583,7 @@
       </c>
       <c r="O9" s="15" t="n">
         <f aca="false">SUM(C9:N9)</f>
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="P9" s="29"/>
     </row>
@@ -3647,7 +3647,7 @@
         <v>0</v>
       </c>
       <c r="D11" s="23" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E11" s="23" t="n">
         <v>1</v>
@@ -3656,13 +3656,13 @@
         <v>1</v>
       </c>
       <c r="G11" s="23" t="n">
+        <v>2</v>
+      </c>
+      <c r="H11" s="23" t="n">
         <v>1</v>
       </c>
-      <c r="H11" s="23" t="n">
+      <c r="I11" s="23" t="n">
         <v>2</v>
-      </c>
-      <c r="I11" s="23" t="n">
-        <v>1</v>
       </c>
       <c r="J11" s="23" t="n">
         <v>2</v>
@@ -3681,7 +3681,7 @@
       </c>
       <c r="O11" s="15" t="n">
         <f aca="false">SUM(C11:N11)</f>
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="P11" s="29"/>
     </row>
@@ -3696,7 +3696,7 @@
         <v>0</v>
       </c>
       <c r="D12" s="23" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E12" s="23" t="n">
         <v>1</v>
@@ -3714,13 +3714,13 @@
         <v>1</v>
       </c>
       <c r="J12" s="23" t="n">
+        <v>2</v>
+      </c>
+      <c r="K12" s="23" t="n">
         <v>1</v>
       </c>
-      <c r="K12" s="23" t="n">
+      <c r="L12" s="23" t="n">
         <v>2</v>
-      </c>
-      <c r="L12" s="23" t="n">
-        <v>1</v>
       </c>
       <c r="M12" s="23" t="n">
         <v>2</v>
@@ -3730,7 +3730,7 @@
       </c>
       <c r="O12" s="15" t="n">
         <f aca="false">SUM(C12:N12)</f>
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="P12" s="29"/>
     </row>
@@ -3815,15 +3815,15 @@
       </c>
       <c r="D16" s="14" t="n">
         <f aca="false">CHOOSE(Assumptions!$B$4,D5,D8,D11)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E16" s="14" t="n">
         <f aca="false">CHOOSE(Assumptions!$B$4,E5,E8,E11)</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F16" s="14" t="n">
         <f aca="false">CHOOSE(Assumptions!$B$4,F5,F8,F11)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G16" s="14" t="n">
         <f aca="false">CHOOSE(Assumptions!$B$4,G5,G8,G11)</f>
@@ -3859,7 +3859,7 @@
       </c>
       <c r="O16" s="15" t="n">
         <f aca="false">SUM(C16:N16)</f>
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3879,23 +3879,23 @@
       </c>
       <c r="E17" s="14" t="n">
         <f aca="false">CHOOSE(Assumptions!$B$4,E6,E9,E12)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F17" s="14" t="n">
         <f aca="false">CHOOSE(Assumptions!$B$4,F6,F9,F12)</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G17" s="14" t="n">
         <f aca="false">CHOOSE(Assumptions!$B$4,G6,G9,G12)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H17" s="14" t="n">
         <f aca="false">CHOOSE(Assumptions!$B$4,H6,H9,H12)</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I17" s="14" t="n">
         <f aca="false">CHOOSE(Assumptions!$B$4,I6,I9,I12)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J17" s="14" t="n">
         <f aca="false">CHOOSE(Assumptions!$B$4,J6,J9,J12)</f>
@@ -3903,11 +3903,11 @@
       </c>
       <c r="K17" s="14" t="n">
         <f aca="false">CHOOSE(Assumptions!$B$4,K6,K9,K12)</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L17" s="14" t="n">
         <f aca="false">CHOOSE(Assumptions!$B$4,L6,L9,L12)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M17" s="14" t="n">
         <f aca="false">CHOOSE(Assumptions!$B$4,M6,M9,M12)</f>
@@ -3919,7 +3919,7 @@
       </c>
       <c r="O17" s="15" t="n">
         <f aca="false">SUM(C17:N17)</f>
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4718,39 +4718,39 @@
       </c>
       <c r="E7" s="9" t="n">
         <f aca="false">INDEX('Sales Plan'!$C$16:$N$16,1,E$4)/3</f>
-        <v>0</v>
+        <v>0.333333333333333</v>
       </c>
       <c r="F7" s="9" t="n">
         <f aca="false">INDEX('Sales Plan'!$C$16:$N$16,1,F$4)/3</f>
-        <v>0</v>
+        <v>0.333333333333333</v>
       </c>
       <c r="G7" s="9" t="n">
         <f aca="false">INDEX('Sales Plan'!$C$16:$N$16,1,G$4)/3</f>
-        <v>0</v>
+        <v>0.333333333333333</v>
       </c>
       <c r="H7" s="9" t="n">
         <f aca="false">INDEX('Sales Plan'!$C$16:$N$16,1,H$4)/3</f>
-        <v>0.333333333333333</v>
+        <v>0</v>
       </c>
       <c r="I7" s="9" t="n">
         <f aca="false">INDEX('Sales Plan'!$C$16:$N$16,1,I$4)/3</f>
-        <v>0.333333333333333</v>
+        <v>0</v>
       </c>
       <c r="J7" s="9" t="n">
         <f aca="false">INDEX('Sales Plan'!$C$16:$N$16,1,J$4)/3</f>
-        <v>0.333333333333333</v>
+        <v>0</v>
       </c>
       <c r="K7" s="9" t="n">
         <f aca="false">INDEX('Sales Plan'!$C$16:$N$16,1,K$4)/3</f>
-        <v>0</v>
+        <v>0.333333333333333</v>
       </c>
       <c r="L7" s="9" t="n">
         <f aca="false">INDEX('Sales Plan'!$C$16:$N$16,1,L$4)/3</f>
-        <v>0</v>
+        <v>0.333333333333333</v>
       </c>
       <c r="M7" s="9" t="n">
         <f aca="false">INDEX('Sales Plan'!$C$16:$N$16,1,M$4)/3</f>
-        <v>0</v>
+        <v>0.333333333333333</v>
       </c>
       <c r="N7" s="9" t="n">
         <f aca="false">INDEX('Sales Plan'!$C$16:$N$16,1,N$4)/3</f>
@@ -4879,63 +4879,63 @@
       </c>
       <c r="H8" s="9" t="n">
         <f aca="false">INDEX('Sales Plan'!$C$17:$N$17,1,H$4)/3</f>
-        <v>0</v>
+        <v>0.333333333333333</v>
       </c>
       <c r="I8" s="9" t="n">
         <f aca="false">INDEX('Sales Plan'!$C$17:$N$17,1,I$4)/3</f>
-        <v>0</v>
+        <v>0.333333333333333</v>
       </c>
       <c r="J8" s="9" t="n">
         <f aca="false">INDEX('Sales Plan'!$C$17:$N$17,1,J$4)/3</f>
-        <v>0</v>
+        <v>0.333333333333333</v>
       </c>
       <c r="K8" s="9" t="n">
         <f aca="false">INDEX('Sales Plan'!$C$17:$N$17,1,K$4)/3</f>
-        <v>0.333333333333333</v>
+        <v>0</v>
       </c>
       <c r="L8" s="9" t="n">
         <f aca="false">INDEX('Sales Plan'!$C$17:$N$17,1,L$4)/3</f>
-        <v>0.333333333333333</v>
+        <v>0</v>
       </c>
       <c r="M8" s="9" t="n">
         <f aca="false">INDEX('Sales Plan'!$C$17:$N$17,1,M$4)/3</f>
-        <v>0.333333333333333</v>
+        <v>0</v>
       </c>
       <c r="N8" s="9" t="n">
         <f aca="false">INDEX('Sales Plan'!$C$17:$N$17,1,N$4)/3</f>
-        <v>0</v>
+        <v>0.333333333333333</v>
       </c>
       <c r="O8" s="9" t="n">
         <f aca="false">INDEX('Sales Plan'!$C$17:$N$17,1,O$4)/3</f>
-        <v>0</v>
+        <v>0.333333333333333</v>
       </c>
       <c r="P8" s="9" t="n">
         <f aca="false">INDEX('Sales Plan'!$C$17:$N$17,1,P$4)/3</f>
-        <v>0</v>
+        <v>0.333333333333333</v>
       </c>
       <c r="Q8" s="9" t="n">
         <f aca="false">INDEX('Sales Plan'!$C$17:$N$17,1,Q$4)/3</f>
-        <v>0.333333333333333</v>
+        <v>0</v>
       </c>
       <c r="R8" s="9" t="n">
         <f aca="false">INDEX('Sales Plan'!$C$17:$N$17,1,R$4)/3</f>
-        <v>0.333333333333333</v>
+        <v>0</v>
       </c>
       <c r="S8" s="9" t="n">
         <f aca="false">INDEX('Sales Plan'!$C$17:$N$17,1,S$4)/3</f>
-        <v>0.333333333333333</v>
+        <v>0</v>
       </c>
       <c r="T8" s="9" t="n">
         <f aca="false">INDEX('Sales Plan'!$C$17:$N$17,1,T$4)/3</f>
-        <v>0</v>
+        <v>0.333333333333333</v>
       </c>
       <c r="U8" s="9" t="n">
         <f aca="false">INDEX('Sales Plan'!$C$17:$N$17,1,U$4)/3</f>
-        <v>0</v>
+        <v>0.333333333333333</v>
       </c>
       <c r="V8" s="9" t="n">
         <f aca="false">INDEX('Sales Plan'!$C$17:$N$17,1,V$4)/3</f>
-        <v>0</v>
+        <v>0.333333333333333</v>
       </c>
       <c r="W8" s="9" t="n">
         <f aca="false">INDEX('Sales Plan'!$C$17:$N$17,1,W$4)/3</f>
@@ -4951,27 +4951,27 @@
       </c>
       <c r="Z8" s="9" t="n">
         <f aca="false">INDEX('Sales Plan'!$C$17:$N$17,1,Z$4)/3</f>
-        <v>0.333333333333333</v>
+        <v>0</v>
       </c>
       <c r="AA8" s="9" t="n">
         <f aca="false">INDEX('Sales Plan'!$C$17:$N$17,1,AA$4)/3</f>
-        <v>0.333333333333333</v>
+        <v>0</v>
       </c>
       <c r="AB8" s="9" t="n">
         <f aca="false">INDEX('Sales Plan'!$C$17:$N$17,1,AB$4)/3</f>
-        <v>0.333333333333333</v>
+        <v>0</v>
       </c>
       <c r="AC8" s="9" t="n">
         <f aca="false">INDEX('Sales Plan'!$C$17:$N$17,1,AC$4)/3</f>
-        <v>0</v>
+        <v>0.333333333333333</v>
       </c>
       <c r="AD8" s="9" t="n">
         <f aca="false">INDEX('Sales Plan'!$C$17:$N$17,1,AD$4)/3</f>
-        <v>0</v>
+        <v>0.333333333333333</v>
       </c>
       <c r="AE8" s="9" t="n">
         <f aca="false">INDEX('Sales Plan'!$C$17:$N$17,1,AE$4)/3</f>
-        <v>0</v>
+        <v>0.333333333333333</v>
       </c>
       <c r="AF8" s="9" t="n">
         <f aca="false">INDEX('Sales Plan'!$C$17:$N$17,1,AF$4)/3</f>
@@ -5170,135 +5170,135 @@
       </c>
       <c r="E12" s="18" t="n">
         <f aca="false">D12*(1-Assumptions!$B$25)+E7</f>
-        <v>0</v>
+        <v>0.333333333333333</v>
       </c>
       <c r="F12" s="18" t="n">
         <f aca="false">E12*(1-Assumptions!$B$25)+F7</f>
-        <v>0</v>
+        <v>0.663752796348434</v>
       </c>
       <c r="G12" s="18" t="n">
         <f aca="false">F12*(1-Assumptions!$B$25)+G7</f>
-        <v>0</v>
+        <v>0.991283860965998</v>
       </c>
       <c r="H12" s="18" t="n">
         <f aca="false">G12*(1-Assumptions!$B$25)+H7</f>
-        <v>0.333333333333333</v>
+        <v>0.982618443107763</v>
       </c>
       <c r="I12" s="18" t="n">
         <f aca="false">H12*(1-Assumptions!$B$25)+I7</f>
-        <v>0.663752796348434</v>
+        <v>0.974028774961206</v>
       </c>
       <c r="J12" s="18" t="n">
         <f aca="false">I12*(1-Assumptions!$B$25)+J7</f>
-        <v>0.991283860965998</v>
+        <v>0.965514194351815</v>
       </c>
       <c r="K12" s="18" t="n">
         <f aca="false">J12*(1-Assumptions!$B$25)+K7</f>
-        <v>0.982618443107763</v>
+        <v>1.29040737822689</v>
       </c>
       <c r="L12" s="18" t="n">
         <f aca="false">K12*(1-Assumptions!$B$25)+L7</f>
-        <v>0.974028774961206</v>
+        <v>1.61246047228669</v>
       </c>
       <c r="M12" s="18" t="n">
         <f aca="false">L12*(1-Assumptions!$B$25)+M7</f>
-        <v>0.965514194351815</v>
+        <v>1.93169830349147</v>
       </c>
       <c r="N12" s="18" t="n">
         <f aca="false">M12*(1-Assumptions!$B$25)+N7</f>
-        <v>1.29040737822689</v>
+        <v>2.24814548177383</v>
       </c>
       <c r="O12" s="18" t="n">
         <f aca="false">N12*(1-Assumptions!$B$25)+O7</f>
-        <v>1.61246047228669</v>
+        <v>2.56182640193594</v>
       </c>
       <c r="P12" s="18" t="n">
         <f aca="false">O12*(1-Assumptions!$B$25)+P7</f>
-        <v>1.93169830349147</v>
+        <v>2.87276524553008</v>
       </c>
       <c r="Q12" s="18" t="n">
         <f aca="false">P12*(1-Assumptions!$B$25)+Q7</f>
-        <v>2.24814548177383</v>
+        <v>3.18098598272281</v>
       </c>
       <c r="R12" s="18" t="n">
         <f aca="false">Q12*(1-Assumptions!$B$25)+R7</f>
-        <v>2.56182640193594</v>
+        <v>3.48651237414284</v>
       </c>
       <c r="S12" s="18" t="n">
         <f aca="false">R12*(1-Assumptions!$B$25)+S7</f>
-        <v>2.87276524553008</v>
+        <v>3.78936797271268</v>
       </c>
       <c r="T12" s="18" t="n">
         <f aca="false">S12*(1-Assumptions!$B$25)+T7</f>
-        <v>3.18098598272281</v>
+        <v>4.08957612546437</v>
       </c>
       <c r="U12" s="18" t="n">
         <f aca="false">T12*(1-Assumptions!$B$25)+U7</f>
-        <v>3.48651237414284</v>
+        <v>4.38715997533928</v>
       </c>
       <c r="V12" s="18" t="n">
         <f aca="false">U12*(1-Assumptions!$B$25)+V7</f>
-        <v>3.78936797271268</v>
+        <v>4.68214246297218</v>
       </c>
       <c r="W12" s="18" t="n">
         <f aca="false">V12*(1-Assumptions!$B$25)+W7</f>
-        <v>4.08957612546437</v>
+        <v>4.97454632845975</v>
       </c>
       <c r="X12" s="18" t="n">
         <f aca="false">W12*(1-Assumptions!$B$25)+X7</f>
-        <v>4.38715997533928</v>
+        <v>5.26439411311357</v>
       </c>
       <c r="Y12" s="18" t="n">
         <f aca="false">X12*(1-Assumptions!$B$25)+Y7</f>
-        <v>4.68214246297218</v>
+        <v>5.55170816119787</v>
       </c>
       <c r="Z12" s="18" t="n">
         <f aca="false">Y12*(1-Assumptions!$B$25)+Z7</f>
-        <v>4.97454632845975</v>
+        <v>5.83651062165199</v>
       </c>
       <c r="AA12" s="18" t="n">
         <f aca="false">Z12*(1-Assumptions!$B$25)+AA7</f>
-        <v>5.26439411311357</v>
+        <v>6.11882344979789</v>
       </c>
       <c r="AB12" s="18" t="n">
         <f aca="false">AA12*(1-Assumptions!$B$25)+AB7</f>
-        <v>5.55170816119787</v>
+        <v>6.39866840903261</v>
       </c>
       <c r="AC12" s="18" t="n">
         <f aca="false">AB12*(1-Assumptions!$B$25)+AC7</f>
-        <v>5.83651062165199</v>
+        <v>6.67606707250608</v>
       </c>
       <c r="AD12" s="18" t="n">
         <f aca="false">AC12*(1-Assumptions!$B$25)+AD7</f>
-        <v>6.11882344979789</v>
+        <v>6.9510408247841</v>
       </c>
       <c r="AE12" s="18" t="n">
         <f aca="false">AD12*(1-Assumptions!$B$25)+AE7</f>
-        <v>6.39866840903261</v>
+        <v>7.22361086349696</v>
       </c>
       <c r="AF12" s="18" t="n">
         <f aca="false">AE12*(1-Assumptions!$B$25)+AF7</f>
-        <v>6.67606707250608</v>
+        <v>7.49379820097348</v>
       </c>
       <c r="AG12" s="18" t="n">
         <f aca="false">AF12*(1-Assumptions!$B$25)+AG7</f>
-        <v>6.9510408247841</v>
+        <v>7.76162366586089</v>
       </c>
       <c r="AH12" s="18" t="n">
         <f aca="false">AG12*(1-Assumptions!$B$25)+AH7</f>
-        <v>7.22361086349696</v>
+        <v>8.02710790473051</v>
       </c>
       <c r="AI12" s="18" t="n">
         <f aca="false">AH12*(1-Assumptions!$B$25)+AI7</f>
-        <v>7.49379820097348</v>
+        <v>8.29027138366931</v>
       </c>
       <c r="AJ12" s="18" t="n">
         <f aca="false">AI12*(1-Assumptions!$B$25)+AJ7</f>
-        <v>7.76162366586089</v>
+        <v>8.55113438985776</v>
       </c>
       <c r="AK12" s="18" t="n">
         <f aca="false">AJ12*(1-Assumptions!$B$25)+AK7</f>
-        <v>8.02710790473051</v>
+        <v>8.80971703313363</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5331,123 +5331,123 @@
       </c>
       <c r="H13" s="18" t="n">
         <f aca="false">G13*(1-Assumptions!$B$25)+H8</f>
-        <v>0</v>
+        <v>0.333333333333333</v>
       </c>
       <c r="I13" s="18" t="n">
         <f aca="false">H13*(1-Assumptions!$B$25)+I8</f>
-        <v>0</v>
+        <v>0.663752796348434</v>
       </c>
       <c r="J13" s="18" t="n">
         <f aca="false">I13*(1-Assumptions!$B$25)+J8</f>
-        <v>0</v>
+        <v>0.991283860965998</v>
       </c>
       <c r="K13" s="18" t="n">
         <f aca="false">J13*(1-Assumptions!$B$25)+K8</f>
-        <v>0.333333333333333</v>
+        <v>0.982618443107763</v>
       </c>
       <c r="L13" s="18" t="n">
         <f aca="false">K13*(1-Assumptions!$B$25)+L8</f>
-        <v>0.663752796348434</v>
+        <v>0.974028774961206</v>
       </c>
       <c r="M13" s="18" t="n">
         <f aca="false">L13*(1-Assumptions!$B$25)+M8</f>
-        <v>0.991283860965998</v>
+        <v>0.965514194351815</v>
       </c>
       <c r="N13" s="18" t="n">
         <f aca="false">M13*(1-Assumptions!$B$25)+N8</f>
-        <v>0.982618443107763</v>
+        <v>1.29040737822689</v>
       </c>
       <c r="O13" s="18" t="n">
         <f aca="false">N13*(1-Assumptions!$B$25)+O8</f>
-        <v>0.974028774961206</v>
+        <v>1.61246047228669</v>
       </c>
       <c r="P13" s="18" t="n">
         <f aca="false">O13*(1-Assumptions!$B$25)+P8</f>
-        <v>0.965514194351815</v>
+        <v>1.93169830349147</v>
       </c>
       <c r="Q13" s="18" t="n">
         <f aca="false">P13*(1-Assumptions!$B$25)+Q8</f>
-        <v>1.29040737822689</v>
+        <v>1.9148121484405</v>
       </c>
       <c r="R13" s="18" t="n">
         <f aca="false">Q13*(1-Assumptions!$B$25)+R8</f>
-        <v>1.61246047228669</v>
+        <v>1.8980736055875</v>
       </c>
       <c r="S13" s="18" t="n">
         <f aca="false">R13*(1-Assumptions!$B$25)+S8</f>
-        <v>1.93169830349147</v>
+        <v>1.88148138456408</v>
       </c>
       <c r="T13" s="18" t="n">
         <f aca="false">S13*(1-Assumptions!$B$25)+T8</f>
-        <v>1.9148121484405</v>
+        <v>2.19836753961505</v>
       </c>
       <c r="U13" s="18" t="n">
         <f aca="false">T13*(1-Assumptions!$B$25)+U8</f>
-        <v>1.8980736055875</v>
+        <v>2.51248359918163</v>
       </c>
       <c r="V13" s="18" t="n">
         <f aca="false">U13*(1-Assumptions!$B$25)+V8</f>
-        <v>1.88148138456408</v>
+        <v>2.82385377836087</v>
       </c>
       <c r="W13" s="18" t="n">
         <f aca="false">V13*(1-Assumptions!$B$25)+W8</f>
-        <v>2.19836753961505</v>
+        <v>3.13250208057082</v>
       </c>
       <c r="X13" s="18" t="n">
         <f aca="false">W13*(1-Assumptions!$B$25)+X8</f>
-        <v>2.51248359918163</v>
+        <v>3.43845229940102</v>
       </c>
       <c r="Y13" s="18" t="n">
         <f aca="false">X13*(1-Assumptions!$B$25)+Y8</f>
-        <v>2.82385377836087</v>
+        <v>3.74172802044671</v>
       </c>
       <c r="Z13" s="18" t="n">
         <f aca="false">Y13*(1-Assumptions!$B$25)+Z8</f>
-        <v>3.13250208057082</v>
+        <v>3.70901928979368</v>
       </c>
       <c r="AA13" s="18" t="n">
         <f aca="false">Z13*(1-Assumptions!$B$25)+AA8</f>
-        <v>3.43845229940102</v>
+        <v>3.67659648613884</v>
       </c>
       <c r="AB13" s="18" t="n">
         <f aca="false">AA13*(1-Assumptions!$B$25)+AB8</f>
-        <v>3.74172802044671</v>
+        <v>3.64445711001961</v>
       </c>
       <c r="AC13" s="18" t="n">
         <f aca="false">AB13*(1-Assumptions!$B$25)+AC8</f>
-        <v>3.70901928979368</v>
+        <v>3.94593201715607</v>
       </c>
       <c r="AD13" s="18" t="n">
         <f aca="false">AC13*(1-Assumptions!$B$25)+AD8</f>
-        <v>3.67659648613884</v>
+        <v>4.24477154794174</v>
       </c>
       <c r="AE13" s="18" t="n">
         <f aca="false">AD13*(1-Assumptions!$B$25)+AE8</f>
-        <v>3.64445711001961</v>
+        <v>4.5409987398114</v>
       </c>
       <c r="AF13" s="18" t="n">
         <f aca="false">AE13*(1-Assumptions!$B$25)+AF8</f>
-        <v>3.94593201715607</v>
+        <v>4.83463642881554</v>
       </c>
       <c r="AG13" s="18" t="n">
         <f aca="false">AF13*(1-Assumptions!$B$25)+AG8</f>
-        <v>4.24477154794174</v>
+        <v>5.12570725138076</v>
       </c>
       <c r="AH13" s="18" t="n">
         <f aca="false">AG13*(1-Assumptions!$B$25)+AH8</f>
-        <v>4.5409987398114</v>
+        <v>5.41423364605485</v>
       </c>
       <c r="AI13" s="18" t="n">
         <f aca="false">AH13*(1-Assumptions!$B$25)+AI8</f>
-        <v>4.83463642881554</v>
+        <v>5.70023785523655</v>
       </c>
       <c r="AJ13" s="18" t="n">
         <f aca="false">AI13*(1-Assumptions!$B$25)+AJ8</f>
-        <v>5.12570725138076</v>
+        <v>5.98374192689017</v>
       </c>
       <c r="AK13" s="18" t="n">
         <f aca="false">AJ13*(1-Assumptions!$B$25)+AK8</f>
-        <v>5.41423364605485</v>
+        <v>6.26476771624532</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5617,135 +5617,135 @@
       </c>
       <c r="E15" s="32" t="n">
         <f aca="false">SUM(E12:E14)</f>
-        <v>0</v>
+        <v>0.333333333333333</v>
       </c>
       <c r="F15" s="32" t="n">
         <f aca="false">SUM(F12:F14)</f>
-        <v>0</v>
+        <v>0.663752796348434</v>
       </c>
       <c r="G15" s="32" t="n">
         <f aca="false">SUM(G12:G14)</f>
-        <v>0</v>
+        <v>0.991283860965998</v>
       </c>
       <c r="H15" s="32" t="n">
         <f aca="false">SUM(H12:H14)</f>
-        <v>0.333333333333333</v>
+        <v>1.3159517764411</v>
       </c>
       <c r="I15" s="32" t="n">
         <f aca="false">SUM(I12:I14)</f>
-        <v>0.663752796348434</v>
+        <v>1.63778157130964</v>
       </c>
       <c r="J15" s="32" t="n">
         <f aca="false">SUM(J12:J14)</f>
-        <v>0.991283860965998</v>
+        <v>1.95679805531781</v>
       </c>
       <c r="K15" s="32" t="n">
         <f aca="false">SUM(K12:K14)</f>
-        <v>1.3159517764411</v>
+        <v>2.27302582133465</v>
       </c>
       <c r="L15" s="32" t="n">
         <f aca="false">SUM(L12:L14)</f>
-        <v>1.63778157130964</v>
+        <v>2.5864892472479</v>
       </c>
       <c r="M15" s="32" t="n">
         <f aca="false">SUM(M12:M14)</f>
-        <v>1.95679805531781</v>
+        <v>2.89721249784328</v>
       </c>
       <c r="N15" s="32" t="n">
         <f aca="false">SUM(N12:N14)</f>
-        <v>2.27302582133465</v>
+        <v>3.53855286000072</v>
       </c>
       <c r="O15" s="32" t="n">
         <f aca="false">SUM(O12:O14)</f>
-        <v>2.5864892472479</v>
+        <v>4.17428687422263</v>
       </c>
       <c r="P15" s="32" t="n">
         <f aca="false">SUM(P12:P14)</f>
-        <v>2.89721249784328</v>
+        <v>4.80446354902155</v>
       </c>
       <c r="Q15" s="32" t="n">
         <f aca="false">SUM(Q12:Q14)</f>
-        <v>3.53855286000072</v>
+        <v>5.09579813116331</v>
       </c>
       <c r="R15" s="32" t="n">
         <f aca="false">SUM(R12:R14)</f>
-        <v>4.17428687422263</v>
+        <v>5.38458597973034</v>
       </c>
       <c r="S15" s="32" t="n">
         <f aca="false">SUM(S12:S14)</f>
-        <v>4.80446354902155</v>
+        <v>5.67084935727676</v>
       </c>
       <c r="T15" s="32" t="n">
         <f aca="false">SUM(T12:T14)</f>
-        <v>5.09579813116331</v>
+        <v>6.28794366507942</v>
       </c>
       <c r="U15" s="32" t="n">
         <f aca="false">SUM(U12:U14)</f>
-        <v>5.38458597973034</v>
+        <v>6.89964357452091</v>
       </c>
       <c r="V15" s="32" t="n">
         <f aca="false">SUM(V12:V14)</f>
-        <v>5.67084935727676</v>
+        <v>7.50599624133305</v>
       </c>
       <c r="W15" s="32" t="n">
         <f aca="false">SUM(W12:W14)</f>
-        <v>6.28794366507942</v>
+        <v>8.10704840903056</v>
       </c>
       <c r="X15" s="32" t="n">
         <f aca="false">SUM(X12:X14)</f>
-        <v>6.89964357452091</v>
+        <v>8.70284641251459</v>
       </c>
       <c r="Y15" s="32" t="n">
         <f aca="false">SUM(Y12:Y14)</f>
-        <v>7.50599624133305</v>
+        <v>9.29343618164458</v>
       </c>
       <c r="Z15" s="32" t="n">
         <f aca="false">SUM(Z12:Z14)</f>
-        <v>8.10704840903056</v>
+        <v>9.54552991144567</v>
       </c>
       <c r="AA15" s="32" t="n">
         <f aca="false">SUM(AA12:AA14)</f>
-        <v>8.70284641251459</v>
+        <v>9.79541993593672</v>
       </c>
       <c r="AB15" s="32" t="n">
         <f aca="false">SUM(AB12:AB14)</f>
-        <v>9.29343618164458</v>
+        <v>10.0431255190522</v>
       </c>
       <c r="AC15" s="32" t="n">
         <f aca="false">SUM(AC12:AC14)</f>
-        <v>9.54552991144567</v>
+        <v>10.6219990896621</v>
       </c>
       <c r="AD15" s="32" t="n">
         <f aca="false">SUM(AD12:AD14)</f>
-        <v>9.79541993593672</v>
+        <v>11.1958123727258</v>
       </c>
       <c r="AE15" s="32" t="n">
         <f aca="false">SUM(AE12:AE14)</f>
-        <v>10.0431255190522</v>
+        <v>11.7646096033084</v>
       </c>
       <c r="AF15" s="32" t="n">
         <f aca="false">SUM(AF12:AF14)</f>
-        <v>10.6219990896621</v>
+        <v>12.328434629789</v>
       </c>
       <c r="AG15" s="32" t="n">
         <f aca="false">SUM(AG12:AG14)</f>
-        <v>11.1958123727258</v>
+        <v>12.8873309172417</v>
       </c>
       <c r="AH15" s="32" t="n">
         <f aca="false">SUM(AH12:AH14)</f>
-        <v>11.7646096033084</v>
+        <v>13.4413415507854</v>
       </c>
       <c r="AI15" s="32" t="n">
         <f aca="false">SUM(AI12:AI14)</f>
-        <v>12.328434629789</v>
+        <v>13.9905092389059</v>
       </c>
       <c r="AJ15" s="32" t="n">
         <f aca="false">SUM(AJ12:AJ14)</f>
-        <v>12.8873309172417</v>
+        <v>14.5348763167479</v>
       </c>
       <c r="AK15" s="32" t="n">
         <f aca="false">SUM(AK12:AK14)</f>
-        <v>13.4413415507854</v>
+        <v>15.0744847493789</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5771,75 +5771,75 @@
       </c>
       <c r="E18" s="17" t="n">
         <f aca="false">(E7*Assumptions!$B$20+E8*Assumptions!$C$20+E9*Assumptions!$D$20)*Assumptions!$B$5</f>
-        <v>0</v>
+        <v>2107.95</v>
       </c>
       <c r="F18" s="17" t="n">
         <f aca="false">(F7*Assumptions!$B$20+F8*Assumptions!$C$20+F9*Assumptions!$D$20)*Assumptions!$B$5</f>
-        <v>0</v>
+        <v>2107.95</v>
       </c>
       <c r="G18" s="17" t="n">
         <f aca="false">(G7*Assumptions!$B$20+G8*Assumptions!$C$20+G9*Assumptions!$D$20)*Assumptions!$B$5</f>
-        <v>0</v>
+        <v>2107.95</v>
       </c>
       <c r="H18" s="17" t="n">
         <f aca="false">(H7*Assumptions!$B$20+H8*Assumptions!$C$20+H9*Assumptions!$D$20)*Assumptions!$B$5</f>
-        <v>2107.95</v>
+        <v>8559.06666666667</v>
       </c>
       <c r="I18" s="17" t="n">
         <f aca="false">(I7*Assumptions!$B$20+I8*Assumptions!$C$20+I9*Assumptions!$D$20)*Assumptions!$B$5</f>
-        <v>2107.95</v>
+        <v>8559.06666666667</v>
       </c>
       <c r="J18" s="17" t="n">
         <f aca="false">(J7*Assumptions!$B$20+J8*Assumptions!$C$20+J9*Assumptions!$D$20)*Assumptions!$B$5</f>
-        <v>2107.95</v>
+        <v>8559.06666666667</v>
       </c>
       <c r="K18" s="17" t="n">
         <f aca="false">(K7*Assumptions!$B$20+K8*Assumptions!$C$20+K9*Assumptions!$D$20)*Assumptions!$B$5</f>
-        <v>8559.06666666667</v>
+        <v>2107.95</v>
       </c>
       <c r="L18" s="17" t="n">
         <f aca="false">(L7*Assumptions!$B$20+L8*Assumptions!$C$20+L9*Assumptions!$D$20)*Assumptions!$B$5</f>
-        <v>8559.06666666667</v>
+        <v>2107.95</v>
       </c>
       <c r="M18" s="17" t="n">
         <f aca="false">(M7*Assumptions!$B$20+M8*Assumptions!$C$20+M9*Assumptions!$D$20)*Assumptions!$B$5</f>
-        <v>8559.06666666667</v>
+        <v>2107.95</v>
       </c>
       <c r="N18" s="17" t="n">
         <f aca="false">(N7*Assumptions!$B$20+N8*Assumptions!$C$20+N9*Assumptions!$D$20)*Assumptions!$B$5</f>
-        <v>2107.95</v>
+        <v>10667.0166666667</v>
       </c>
       <c r="O18" s="17" t="n">
         <f aca="false">(O7*Assumptions!$B$20+O8*Assumptions!$C$20+O9*Assumptions!$D$20)*Assumptions!$B$5</f>
-        <v>2107.95</v>
+        <v>10667.0166666667</v>
       </c>
       <c r="P18" s="17" t="n">
         <f aca="false">(P7*Assumptions!$B$20+P8*Assumptions!$C$20+P9*Assumptions!$D$20)*Assumptions!$B$5</f>
-        <v>2107.95</v>
+        <v>10667.0166666667</v>
       </c>
       <c r="Q18" s="17" t="n">
         <f aca="false">(Q7*Assumptions!$B$20+Q8*Assumptions!$C$20+Q9*Assumptions!$D$20)*Assumptions!$B$5</f>
-        <v>10667.0166666667</v>
+        <v>2107.95</v>
       </c>
       <c r="R18" s="17" t="n">
         <f aca="false">(R7*Assumptions!$B$20+R8*Assumptions!$C$20+R9*Assumptions!$D$20)*Assumptions!$B$5</f>
-        <v>10667.0166666667</v>
+        <v>2107.95</v>
       </c>
       <c r="S18" s="17" t="n">
         <f aca="false">(S7*Assumptions!$B$20+S8*Assumptions!$C$20+S9*Assumptions!$D$20)*Assumptions!$B$5</f>
-        <v>10667.0166666667</v>
+        <v>2107.95</v>
       </c>
       <c r="T18" s="17" t="n">
         <f aca="false">(T7*Assumptions!$B$20+T8*Assumptions!$C$20+T9*Assumptions!$D$20)*Assumptions!$B$5</f>
-        <v>2107.95</v>
+        <v>10667.0166666667</v>
       </c>
       <c r="U18" s="17" t="n">
         <f aca="false">(U7*Assumptions!$B$20+U8*Assumptions!$C$20+U9*Assumptions!$D$20)*Assumptions!$B$5</f>
-        <v>2107.95</v>
+        <v>10667.0166666667</v>
       </c>
       <c r="V18" s="17" t="n">
         <f aca="false">(V7*Assumptions!$B$20+V8*Assumptions!$C$20+V9*Assumptions!$D$20)*Assumptions!$B$5</f>
-        <v>2107.95</v>
+        <v>10667.0166666667</v>
       </c>
       <c r="W18" s="17" t="n">
         <f aca="false">(W7*Assumptions!$B$20+W8*Assumptions!$C$20+W9*Assumptions!$D$20)*Assumptions!$B$5</f>
@@ -5855,27 +5855,27 @@
       </c>
       <c r="Z18" s="17" t="n">
         <f aca="false">(Z7*Assumptions!$B$20+Z8*Assumptions!$C$20+Z9*Assumptions!$D$20)*Assumptions!$B$5</f>
-        <v>10667.0166666667</v>
+        <v>2107.95</v>
       </c>
       <c r="AA18" s="17" t="n">
         <f aca="false">(AA7*Assumptions!$B$20+AA8*Assumptions!$C$20+AA9*Assumptions!$D$20)*Assumptions!$B$5</f>
-        <v>10667.0166666667</v>
+        <v>2107.95</v>
       </c>
       <c r="AB18" s="17" t="n">
         <f aca="false">(AB7*Assumptions!$B$20+AB8*Assumptions!$C$20+AB9*Assumptions!$D$20)*Assumptions!$B$5</f>
-        <v>10667.0166666667</v>
+        <v>2107.95</v>
       </c>
       <c r="AC18" s="17" t="n">
         <f aca="false">(AC7*Assumptions!$B$20+AC8*Assumptions!$C$20+AC9*Assumptions!$D$20)*Assumptions!$B$5</f>
-        <v>2107.95</v>
+        <v>10667.0166666667</v>
       </c>
       <c r="AD18" s="17" t="n">
         <f aca="false">(AD7*Assumptions!$B$20+AD8*Assumptions!$C$20+AD9*Assumptions!$D$20)*Assumptions!$B$5</f>
-        <v>2107.95</v>
+        <v>10667.0166666667</v>
       </c>
       <c r="AE18" s="17" t="n">
         <f aca="false">(AE7*Assumptions!$B$20+AE8*Assumptions!$C$20+AE9*Assumptions!$D$20)*Assumptions!$B$5</f>
-        <v>2107.95</v>
+        <v>10667.0166666667</v>
       </c>
       <c r="AF18" s="17" t="n">
         <f aca="false">(AF7*Assumptions!$B$20+AF8*Assumptions!$C$20+AF9*Assumptions!$D$20)*Assumptions!$B$5</f>
@@ -5920,75 +5920,75 @@
       </c>
       <c r="E19" s="17" t="n">
         <f aca="false">E7*Assumptions!$B$11+E8*Assumptions!$C$11+E9*Assumptions!$D$11</f>
-        <v>0</v>
+        <v>1500</v>
       </c>
       <c r="F19" s="17" t="n">
         <f aca="false">F7*Assumptions!$B$11+F8*Assumptions!$C$11+F9*Assumptions!$D$11</f>
-        <v>0</v>
+        <v>1500</v>
       </c>
       <c r="G19" s="17" t="n">
         <f aca="false">G7*Assumptions!$B$11+G8*Assumptions!$C$11+G9*Assumptions!$D$11</f>
-        <v>0</v>
+        <v>1500</v>
       </c>
       <c r="H19" s="17" t="n">
         <f aca="false">H7*Assumptions!$B$11+H8*Assumptions!$C$11+H9*Assumptions!$D$11</f>
-        <v>1500</v>
+        <v>4000</v>
       </c>
       <c r="I19" s="17" t="n">
         <f aca="false">I7*Assumptions!$B$11+I8*Assumptions!$C$11+I9*Assumptions!$D$11</f>
-        <v>1500</v>
+        <v>4000</v>
       </c>
       <c r="J19" s="17" t="n">
         <f aca="false">J7*Assumptions!$B$11+J8*Assumptions!$C$11+J9*Assumptions!$D$11</f>
-        <v>1500</v>
+        <v>4000</v>
       </c>
       <c r="K19" s="17" t="n">
         <f aca="false">K7*Assumptions!$B$11+K8*Assumptions!$C$11+K9*Assumptions!$D$11</f>
-        <v>4000</v>
+        <v>1500</v>
       </c>
       <c r="L19" s="17" t="n">
         <f aca="false">L7*Assumptions!$B$11+L8*Assumptions!$C$11+L9*Assumptions!$D$11</f>
-        <v>4000</v>
+        <v>1500</v>
       </c>
       <c r="M19" s="17" t="n">
         <f aca="false">M7*Assumptions!$B$11+M8*Assumptions!$C$11+M9*Assumptions!$D$11</f>
-        <v>4000</v>
+        <v>1500</v>
       </c>
       <c r="N19" s="17" t="n">
         <f aca="false">N7*Assumptions!$B$11+N8*Assumptions!$C$11+N9*Assumptions!$D$11</f>
-        <v>1500</v>
+        <v>5500</v>
       </c>
       <c r="O19" s="17" t="n">
         <f aca="false">O7*Assumptions!$B$11+O8*Assumptions!$C$11+O9*Assumptions!$D$11</f>
-        <v>1500</v>
+        <v>5500</v>
       </c>
       <c r="P19" s="17" t="n">
         <f aca="false">P7*Assumptions!$B$11+P8*Assumptions!$C$11+P9*Assumptions!$D$11</f>
-        <v>1500</v>
+        <v>5500</v>
       </c>
       <c r="Q19" s="17" t="n">
         <f aca="false">Q7*Assumptions!$B$11+Q8*Assumptions!$C$11+Q9*Assumptions!$D$11</f>
-        <v>5500</v>
+        <v>1500</v>
       </c>
       <c r="R19" s="17" t="n">
         <f aca="false">R7*Assumptions!$B$11+R8*Assumptions!$C$11+R9*Assumptions!$D$11</f>
-        <v>5500</v>
+        <v>1500</v>
       </c>
       <c r="S19" s="17" t="n">
         <f aca="false">S7*Assumptions!$B$11+S8*Assumptions!$C$11+S9*Assumptions!$D$11</f>
-        <v>5500</v>
+        <v>1500</v>
       </c>
       <c r="T19" s="17" t="n">
         <f aca="false">T7*Assumptions!$B$11+T8*Assumptions!$C$11+T9*Assumptions!$D$11</f>
-        <v>1500</v>
+        <v>5500</v>
       </c>
       <c r="U19" s="17" t="n">
         <f aca="false">U7*Assumptions!$B$11+U8*Assumptions!$C$11+U9*Assumptions!$D$11</f>
-        <v>1500</v>
+        <v>5500</v>
       </c>
       <c r="V19" s="17" t="n">
         <f aca="false">V7*Assumptions!$B$11+V8*Assumptions!$C$11+V9*Assumptions!$D$11</f>
-        <v>1500</v>
+        <v>5500</v>
       </c>
       <c r="W19" s="17" t="n">
         <f aca="false">W7*Assumptions!$B$11+W8*Assumptions!$C$11+W9*Assumptions!$D$11</f>
@@ -6004,27 +6004,27 @@
       </c>
       <c r="Z19" s="17" t="n">
         <f aca="false">Z7*Assumptions!$B$11+Z8*Assumptions!$C$11+Z9*Assumptions!$D$11</f>
-        <v>5500</v>
+        <v>1500</v>
       </c>
       <c r="AA19" s="17" t="n">
         <f aca="false">AA7*Assumptions!$B$11+AA8*Assumptions!$C$11+AA9*Assumptions!$D$11</f>
-        <v>5500</v>
+        <v>1500</v>
       </c>
       <c r="AB19" s="17" t="n">
         <f aca="false">AB7*Assumptions!$B$11+AB8*Assumptions!$C$11+AB9*Assumptions!$D$11</f>
-        <v>5500</v>
+        <v>1500</v>
       </c>
       <c r="AC19" s="17" t="n">
         <f aca="false">AC7*Assumptions!$B$11+AC8*Assumptions!$C$11+AC9*Assumptions!$D$11</f>
-        <v>1500</v>
+        <v>5500</v>
       </c>
       <c r="AD19" s="17" t="n">
         <f aca="false">AD7*Assumptions!$B$11+AD8*Assumptions!$C$11+AD9*Assumptions!$D$11</f>
-        <v>1500</v>
+        <v>5500</v>
       </c>
       <c r="AE19" s="17" t="n">
         <f aca="false">AE7*Assumptions!$B$11+AE8*Assumptions!$C$11+AE9*Assumptions!$D$11</f>
-        <v>1500</v>
+        <v>5500</v>
       </c>
       <c r="AF19" s="17" t="n">
         <f aca="false">AF7*Assumptions!$B$11+AF8*Assumptions!$C$11+AF9*Assumptions!$D$11</f>
@@ -6069,135 +6069,135 @@
       </c>
       <c r="E20" s="17" t="n">
         <f aca="false">(E12*Assumptions!$B$12+E13*Assumptions!$C$12+E14*Assumptions!$D$12)*(1-IF(E$3=1,Assumptions!$B$26,0))*(1-Assumptions!$B$31*Assumptions!$B$32)</f>
-        <v>0</v>
+        <v>250</v>
       </c>
       <c r="F20" s="17" t="n">
         <f aca="false">(F12*Assumptions!$B$12+F13*Assumptions!$C$12+F14*Assumptions!$D$12)*(1-IF(F$3=1,Assumptions!$B$26,0))*(1-Assumptions!$B$31*Assumptions!$B$32)</f>
-        <v>0</v>
+        <v>497.814597261326</v>
       </c>
       <c r="G20" s="17" t="n">
         <f aca="false">(G12*Assumptions!$B$12+G13*Assumptions!$C$12+G14*Assumptions!$D$12)*(1-IF(G$3=1,Assumptions!$B$26,0))*(1-Assumptions!$B$31*Assumptions!$B$32)</f>
-        <v>0</v>
+        <v>743.462895724498</v>
       </c>
       <c r="H20" s="17" t="n">
         <f aca="false">(H12*Assumptions!$B$12+H13*Assumptions!$C$12+H14*Assumptions!$D$12)*(1-IF(H$3=1,Assumptions!$B$26,0))*(1-Assumptions!$B$31*Assumptions!$B$32)</f>
-        <v>250</v>
+        <v>1403.63049899749</v>
       </c>
       <c r="I20" s="17" t="n">
         <f aca="false">(I12*Assumptions!$B$12+I13*Assumptions!$C$12+I14*Assumptions!$D$12)*(1-IF(I$3=1,Assumptions!$B$26,0))*(1-Assumptions!$B$31*Assumptions!$B$32)</f>
-        <v>497.814597261326</v>
+        <v>2058.02717391777</v>
       </c>
       <c r="J20" s="17" t="n">
         <f aca="false">(J12*Assumptions!$B$12+J13*Assumptions!$C$12+J14*Assumptions!$D$12)*(1-IF(J$3=1,Assumptions!$B$26,0))*(1-Assumptions!$B$31*Assumptions!$B$32)</f>
-        <v>743.462895724498</v>
+        <v>2706.70336769586</v>
       </c>
       <c r="K20" s="17" t="n">
         <f aca="false">(K12*Assumptions!$B$12+K13*Assumptions!$C$12+K14*Assumptions!$D$12)*(1-IF(K$3=1,Assumptions!$B$26,0))*(1-Assumptions!$B$31*Assumptions!$B$32)</f>
-        <v>1403.63049899749</v>
+        <v>2933.04241988569</v>
       </c>
       <c r="L20" s="17" t="n">
         <f aca="false">(L12*Assumptions!$B$12+L13*Assumptions!$C$12+L14*Assumptions!$D$12)*(1-IF(L$3=1,Assumptions!$B$26,0))*(1-Assumptions!$B$31*Assumptions!$B$32)</f>
-        <v>2058.02717391777</v>
+        <v>3157.40290413743</v>
       </c>
       <c r="M20" s="17" t="n">
         <f aca="false">(M12*Assumptions!$B$12+M13*Assumptions!$C$12+M14*Assumptions!$D$12)*(1-IF(M$3=1,Assumptions!$B$26,0))*(1-Assumptions!$B$31*Assumptions!$B$32)</f>
-        <v>2706.70336769586</v>
+        <v>3379.80211632223</v>
       </c>
       <c r="N20" s="17" t="n">
         <f aca="false">(N12*Assumptions!$B$12+N13*Assumptions!$C$12+N14*Assumptions!$D$12)*(1-IF(N$3=1,Assumptions!$B$26,0))*(1-Assumptions!$B$31*Assumptions!$B$32)</f>
-        <v>5866.08483977138</v>
+        <v>8533.8477355683</v>
       </c>
       <c r="O20" s="17" t="n">
         <f aca="false">(O12*Assumptions!$B$12+O13*Assumptions!$C$12+O14*Assumptions!$D$12)*(1-IF(O$3=1,Assumptions!$B$26,0))*(1-Assumptions!$B$31*Assumptions!$B$32)</f>
-        <v>6314.80580827486</v>
+        <v>10292.5814920507</v>
       </c>
       <c r="P20" s="17" t="n">
         <f aca="false">(P12*Assumptions!$B$12+P13*Assumptions!$C$12+P14*Assumptions!$D$12)*(1-IF(P$3=1,Assumptions!$B$26,0))*(1-Assumptions!$B$31*Assumptions!$B$32)</f>
-        <v>6759.60423264446</v>
+        <v>12035.941082261</v>
       </c>
       <c r="Q20" s="17" t="n">
         <f aca="false">(Q12*Assumptions!$B$12+Q13*Assumptions!$C$12+Q14*Assumptions!$D$12)*(1-IF(Q$3=1,Assumptions!$B$26,0))*(1-Assumptions!$B$31*Assumptions!$B$32)</f>
-        <v>8533.8477355683</v>
+        <v>12430.7275678462</v>
       </c>
       <c r="R20" s="17" t="n">
         <f aca="false">(R12*Assumptions!$B$12+R13*Assumptions!$C$12+R14*Assumptions!$D$12)*(1-IF(R$3=1,Assumptions!$B$26,0))*(1-Assumptions!$B$31*Assumptions!$B$32)</f>
-        <v>10292.5814920507</v>
+        <v>12822.0629835643</v>
       </c>
       <c r="S20" s="17" t="n">
         <f aca="false">(S12*Assumptions!$B$12+S13*Assumptions!$C$12+S14*Assumptions!$D$12)*(1-IF(S$3=1,Assumptions!$B$26,0))*(1-Assumptions!$B$31*Assumptions!$B$32)</f>
-        <v>12035.941082261</v>
+        <v>13209.9774973253</v>
       </c>
       <c r="T20" s="17" t="n">
         <f aca="false">(T12*Assumptions!$B$12+T13*Assumptions!$C$12+T14*Assumptions!$D$12)*(1-IF(T$3=1,Assumptions!$B$26,0))*(1-Assumptions!$B$31*Assumptions!$B$32)</f>
-        <v>12430.7275678462</v>
+        <v>14927.8343466568</v>
       </c>
       <c r="U20" s="17" t="n">
         <f aca="false">(U12*Assumptions!$B$12+U13*Assumptions!$C$12+U14*Assumptions!$D$12)*(1-IF(U$3=1,Assumptions!$B$26,0))*(1-Assumptions!$B$31*Assumptions!$B$32)</f>
-        <v>12822.0629835643</v>
+        <v>16630.6743597355</v>
       </c>
       <c r="V20" s="17" t="n">
         <f aca="false">(V12*Assumptions!$B$12+V13*Assumptions!$C$12+V14*Assumptions!$D$12)*(1-IF(V$3=1,Assumptions!$B$26,0))*(1-Assumptions!$B$31*Assumptions!$B$32)</f>
-        <v>13209.9774973253</v>
+        <v>18318.6288079017</v>
       </c>
       <c r="W20" s="17" t="n">
         <f aca="false">(W12*Assumptions!$B$12+W13*Assumptions!$C$12+W14*Assumptions!$D$12)*(1-IF(W$3=1,Assumptions!$B$26,0))*(1-Assumptions!$B$31*Assumptions!$B$32)</f>
-        <v>14927.8343466568</v>
+        <v>19991.8278149729</v>
       </c>
       <c r="X20" s="17" t="n">
         <f aca="false">(X12*Assumptions!$B$12+X13*Assumptions!$C$12+X14*Assumptions!$D$12)*(1-IF(X$3=1,Assumptions!$B$26,0))*(1-Assumptions!$B$31*Assumptions!$B$32)</f>
-        <v>16630.6743597355</v>
+        <v>21650.4003672744</v>
       </c>
       <c r="Y20" s="17" t="n">
         <f aca="false">(Y12*Assumptions!$B$12+Y13*Assumptions!$C$12+Y14*Assumptions!$D$12)*(1-IF(Y$3=1,Assumptions!$B$26,0))*(1-Assumptions!$B$31*Assumptions!$B$32)</f>
-        <v>18318.6288079017</v>
+        <v>23294.4743235836</v>
       </c>
       <c r="Z20" s="17" t="n">
         <f aca="false">(Z12*Assumptions!$B$12+Z13*Assumptions!$C$12+Z14*Assumptions!$D$12)*(1-IF(Z$3=1,Assumptions!$B$26,0))*(1-Assumptions!$B$31*Assumptions!$B$32)</f>
-        <v>19991.8278149729</v>
+        <v>23590.8430916527</v>
       </c>
       <c r="AA20" s="17" t="n">
         <f aca="false">(AA12*Assumptions!$B$12+AA13*Assumptions!$C$12+AA14*Assumptions!$D$12)*(1-IF(AA$3=1,Assumptions!$B$26,0))*(1-Assumptions!$B$31*Assumptions!$B$32)</f>
-        <v>21650.4003672744</v>
+        <v>23884.6211192522</v>
       </c>
       <c r="AB20" s="17" t="n">
         <f aca="false">(AB12*Assumptions!$B$12+AB13*Assumptions!$C$12+AB14*Assumptions!$D$12)*(1-IF(AB$3=1,Assumptions!$B$26,0))*(1-Assumptions!$B$31*Assumptions!$B$32)</f>
-        <v>23294.4743235836</v>
+        <v>24175.8310536273</v>
       </c>
       <c r="AC20" s="17" t="n">
         <f aca="false">(AC12*Assumptions!$B$12+AC13*Assumptions!$C$12+AC14*Assumptions!$D$12)*(1-IF(AC$3=1,Assumptions!$B$26,0))*(1-Assumptions!$B$31*Assumptions!$B$32)</f>
-        <v>23590.8430916527</v>
+        <v>25797.8286773834</v>
       </c>
       <c r="AD20" s="17" t="n">
         <f aca="false">(AD12*Assumptions!$B$12+AD13*Assumptions!$C$12+AD14*Assumptions!$D$12)*(1-IF(AD$3=1,Assumptions!$B$26,0))*(1-Assumptions!$B$31*Assumptions!$B$32)</f>
-        <v>23884.6211192522</v>
+        <v>27405.6474289431</v>
       </c>
       <c r="AE20" s="17" t="n">
         <f aca="false">(AE12*Assumptions!$B$12+AE13*Assumptions!$C$12+AE14*Assumptions!$D$12)*(1-IF(AE$3=1,Assumptions!$B$26,0))*(1-Assumptions!$B$31*Assumptions!$B$32)</f>
-        <v>24175.8310536273</v>
+        <v>28999.411254491</v>
       </c>
       <c r="AF20" s="17" t="n">
         <f aca="false">(AF12*Assumptions!$B$12+AF13*Assumptions!$C$12+AF14*Assumptions!$D$12)*(1-IF(AF$3=1,Assumptions!$B$26,0))*(1-Assumptions!$B$31*Assumptions!$B$32)</f>
-        <v>25797.8286773834</v>
+        <v>30579.2430167224</v>
       </c>
       <c r="AG20" s="17" t="n">
         <f aca="false">(AG12*Assumptions!$B$12+AG13*Assumptions!$C$12+AG14*Assumptions!$D$12)*(1-IF(AG$3=1,Assumptions!$B$26,0))*(1-Assumptions!$B$31*Assumptions!$B$32)</f>
-        <v>27405.6474289431</v>
+        <v>32145.2645043144</v>
       </c>
       <c r="AH20" s="17" t="n">
         <f aca="false">(AH12*Assumptions!$B$12+AH13*Assumptions!$C$12+AH14*Assumptions!$D$12)*(1-IF(AH$3=1,Assumptions!$B$26,0))*(1-Assumptions!$B$31*Assumptions!$B$32)</f>
-        <v>28999.411254491</v>
+        <v>33697.5964413152</v>
       </c>
       <c r="AI20" s="17" t="n">
         <f aca="false">(AI12*Assumptions!$B$12+AI13*Assumptions!$C$12+AI14*Assumptions!$D$12)*(1-IF(AI$3=1,Assumptions!$B$26,0))*(1-Assumptions!$B$31*Assumptions!$B$32)</f>
-        <v>30579.2430167224</v>
+        <v>35236.3584964502</v>
       </c>
       <c r="AJ20" s="17" t="n">
         <f aca="false">(AJ12*Assumptions!$B$12+AJ13*Assumptions!$C$12+AJ14*Assumptions!$D$12)*(1-IF(AJ$3=1,Assumptions!$B$26,0))*(1-Assumptions!$B$31*Assumptions!$B$32)</f>
-        <v>32145.2645043144</v>
+        <v>36761.6692923473</v>
       </c>
       <c r="AK20" s="17" t="n">
         <f aca="false">(AK12*Assumptions!$B$12+AK13*Assumptions!$C$12+AK14*Assumptions!$D$12)*(1-IF(AK$3=1,Assumptions!$B$26,0))*(1-Assumptions!$B$31*Assumptions!$B$32)</f>
-        <v>33697.5964413152</v>
+        <v>38273.6464146817</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6218,135 +6218,135 @@
       </c>
       <c r="E21" s="12" t="n">
         <f aca="false">SUM(E18:E20)</f>
-        <v>0</v>
+        <v>3857.95</v>
       </c>
       <c r="F21" s="12" t="n">
         <f aca="false">SUM(F18:F20)</f>
-        <v>0</v>
+        <v>4105.76459726133</v>
       </c>
       <c r="G21" s="12" t="n">
         <f aca="false">SUM(G18:G20)</f>
-        <v>0</v>
+        <v>4351.4128957245</v>
       </c>
       <c r="H21" s="12" t="n">
         <f aca="false">SUM(H18:H20)</f>
-        <v>3857.95</v>
+        <v>13962.6971656642</v>
       </c>
       <c r="I21" s="12" t="n">
         <f aca="false">SUM(I18:I20)</f>
-        <v>4105.76459726133</v>
+        <v>14617.0938405844</v>
       </c>
       <c r="J21" s="12" t="n">
         <f aca="false">SUM(J18:J20)</f>
-        <v>4351.4128957245</v>
+        <v>15265.7700343625</v>
       </c>
       <c r="K21" s="12" t="n">
         <f aca="false">SUM(K18:K20)</f>
-        <v>13962.6971656642</v>
+        <v>6540.99241988569</v>
       </c>
       <c r="L21" s="12" t="n">
         <f aca="false">SUM(L18:L20)</f>
-        <v>14617.0938405844</v>
+        <v>6765.35290413743</v>
       </c>
       <c r="M21" s="12" t="n">
         <f aca="false">SUM(M18:M20)</f>
-        <v>15265.7700343625</v>
+        <v>6987.75211632223</v>
       </c>
       <c r="N21" s="12" t="n">
         <f aca="false">SUM(N18:N20)</f>
-        <v>9474.03483977138</v>
+        <v>24700.864402235</v>
       </c>
       <c r="O21" s="12" t="n">
         <f aca="false">SUM(O18:O20)</f>
-        <v>9922.75580827486</v>
+        <v>26459.5981587173</v>
       </c>
       <c r="P21" s="12" t="n">
         <f aca="false">SUM(P18:P20)</f>
-        <v>10367.5542326445</v>
+        <v>28202.9577489277</v>
       </c>
       <c r="Q21" s="12" t="n">
         <f aca="false">SUM(Q18:Q20)</f>
-        <v>24700.864402235</v>
+        <v>16038.6775678462</v>
       </c>
       <c r="R21" s="12" t="n">
         <f aca="false">SUM(R18:R20)</f>
-        <v>26459.5981587173</v>
+        <v>16430.0129835643</v>
       </c>
       <c r="S21" s="12" t="n">
         <f aca="false">SUM(S18:S20)</f>
-        <v>28202.9577489277</v>
+        <v>16817.9274973253</v>
       </c>
       <c r="T21" s="12" t="n">
         <f aca="false">SUM(T18:T20)</f>
-        <v>16038.6775678462</v>
+        <v>31094.8510133234</v>
       </c>
       <c r="U21" s="12" t="n">
         <f aca="false">SUM(U18:U20)</f>
-        <v>16430.0129835643</v>
+        <v>32797.6910264021</v>
       </c>
       <c r="V21" s="12" t="n">
         <f aca="false">SUM(V18:V20)</f>
-        <v>16817.9274973253</v>
+        <v>34485.6454745684</v>
       </c>
       <c r="W21" s="12" t="n">
         <f aca="false">SUM(W18:W20)</f>
-        <v>31094.8510133234</v>
+        <v>36158.8444816396</v>
       </c>
       <c r="X21" s="12" t="n">
         <f aca="false">SUM(X18:X20)</f>
-        <v>32797.6910264021</v>
+        <v>37817.4170339411</v>
       </c>
       <c r="Y21" s="12" t="n">
         <f aca="false">SUM(Y18:Y20)</f>
-        <v>34485.6454745684</v>
+        <v>39461.4909902503</v>
       </c>
       <c r="Z21" s="12" t="n">
         <f aca="false">SUM(Z18:Z20)</f>
-        <v>36158.8444816396</v>
+        <v>27198.7930916527</v>
       </c>
       <c r="AA21" s="12" t="n">
         <f aca="false">SUM(AA18:AA20)</f>
-        <v>37817.4170339411</v>
+        <v>27492.5711192522</v>
       </c>
       <c r="AB21" s="12" t="n">
         <f aca="false">SUM(AB18:AB20)</f>
-        <v>39461.4909902503</v>
+        <v>27783.7810536273</v>
       </c>
       <c r="AC21" s="12" t="n">
         <f aca="false">SUM(AC18:AC20)</f>
-        <v>27198.7930916527</v>
+        <v>41964.8453440501</v>
       </c>
       <c r="AD21" s="12" t="n">
         <f aca="false">SUM(AD18:AD20)</f>
-        <v>27492.5711192522</v>
+        <v>43572.6640956098</v>
       </c>
       <c r="AE21" s="12" t="n">
         <f aca="false">SUM(AE18:AE20)</f>
-        <v>27783.7810536273</v>
+        <v>45166.4279211577</v>
       </c>
       <c r="AF21" s="12" t="n">
         <f aca="false">SUM(AF18:AF20)</f>
-        <v>41964.8453440501</v>
+        <v>46746.259683389</v>
       </c>
       <c r="AG21" s="12" t="n">
         <f aca="false">SUM(AG18:AG20)</f>
-        <v>43572.6640956098</v>
+        <v>48312.2811709811</v>
       </c>
       <c r="AH21" s="12" t="n">
         <f aca="false">SUM(AH18:AH20)</f>
-        <v>45166.4279211577</v>
+        <v>49864.6131079818</v>
       </c>
       <c r="AI21" s="12" t="n">
         <f aca="false">SUM(AI18:AI20)</f>
-        <v>46746.259683389</v>
+        <v>51403.3751631168</v>
       </c>
       <c r="AJ21" s="12" t="n">
         <f aca="false">SUM(AJ18:AJ20)</f>
-        <v>48312.2811709811</v>
+        <v>52928.685959014</v>
       </c>
       <c r="AK21" s="12" t="n">
         <f aca="false">SUM(AK18:AK20)</f>
-        <v>49864.6131079818</v>
+        <v>54440.6630813484</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6372,75 +6372,75 @@
       </c>
       <c r="E24" s="17" t="n">
         <f aca="false">(E7*Assumptions!$B$14+E8*Assumptions!$C$14+E9*Assumptions!$D$14)*Assumptions!$B$5</f>
-        <v>0</v>
+        <v>1833</v>
       </c>
       <c r="F24" s="17" t="n">
         <f aca="false">(F7*Assumptions!$B$14+F8*Assumptions!$C$14+F9*Assumptions!$D$14)*Assumptions!$B$5</f>
-        <v>0</v>
+        <v>1833</v>
       </c>
       <c r="G24" s="17" t="n">
         <f aca="false">(G7*Assumptions!$B$14+G8*Assumptions!$C$14+G9*Assumptions!$D$14)*Assumptions!$B$5</f>
-        <v>0</v>
+        <v>1833</v>
       </c>
       <c r="H24" s="17" t="n">
         <f aca="false">(H7*Assumptions!$B$14+H8*Assumptions!$C$14+H9*Assumptions!$D$14)*Assumptions!$B$5</f>
-        <v>1833</v>
+        <v>7442.66666666667</v>
       </c>
       <c r="I24" s="17" t="n">
         <f aca="false">(I7*Assumptions!$B$14+I8*Assumptions!$C$14+I9*Assumptions!$D$14)*Assumptions!$B$5</f>
-        <v>1833</v>
+        <v>7442.66666666667</v>
       </c>
       <c r="J24" s="17" t="n">
         <f aca="false">(J7*Assumptions!$B$14+J8*Assumptions!$C$14+J9*Assumptions!$D$14)*Assumptions!$B$5</f>
-        <v>1833</v>
+        <v>7442.66666666667</v>
       </c>
       <c r="K24" s="17" t="n">
         <f aca="false">(K7*Assumptions!$B$14+K8*Assumptions!$C$14+K9*Assumptions!$D$14)*Assumptions!$B$5</f>
-        <v>7442.66666666667</v>
+        <v>1833</v>
       </c>
       <c r="L24" s="17" t="n">
         <f aca="false">(L7*Assumptions!$B$14+L8*Assumptions!$C$14+L9*Assumptions!$D$14)*Assumptions!$B$5</f>
-        <v>7442.66666666667</v>
+        <v>1833</v>
       </c>
       <c r="M24" s="17" t="n">
         <f aca="false">(M7*Assumptions!$B$14+M8*Assumptions!$C$14+M9*Assumptions!$D$14)*Assumptions!$B$5</f>
-        <v>7442.66666666667</v>
+        <v>1833</v>
       </c>
       <c r="N24" s="17" t="n">
         <f aca="false">(N7*Assumptions!$B$14+N8*Assumptions!$C$14+N9*Assumptions!$D$14)*Assumptions!$B$5</f>
-        <v>1833</v>
+        <v>9275.66666666667</v>
       </c>
       <c r="O24" s="17" t="n">
         <f aca="false">(O7*Assumptions!$B$14+O8*Assumptions!$C$14+O9*Assumptions!$D$14)*Assumptions!$B$5</f>
-        <v>1833</v>
+        <v>9275.66666666667</v>
       </c>
       <c r="P24" s="17" t="n">
         <f aca="false">(P7*Assumptions!$B$14+P8*Assumptions!$C$14+P9*Assumptions!$D$14)*Assumptions!$B$5</f>
-        <v>1833</v>
+        <v>9275.66666666667</v>
       </c>
       <c r="Q24" s="17" t="n">
         <f aca="false">(Q7*Assumptions!$B$14+Q8*Assumptions!$C$14+Q9*Assumptions!$D$14)*Assumptions!$B$5</f>
-        <v>9275.66666666667</v>
+        <v>1833</v>
       </c>
       <c r="R24" s="17" t="n">
         <f aca="false">(R7*Assumptions!$B$14+R8*Assumptions!$C$14+R9*Assumptions!$D$14)*Assumptions!$B$5</f>
-        <v>9275.66666666667</v>
+        <v>1833</v>
       </c>
       <c r="S24" s="17" t="n">
         <f aca="false">(S7*Assumptions!$B$14+S8*Assumptions!$C$14+S9*Assumptions!$D$14)*Assumptions!$B$5</f>
-        <v>9275.66666666667</v>
+        <v>1833</v>
       </c>
       <c r="T24" s="17" t="n">
         <f aca="false">(T7*Assumptions!$B$14+T8*Assumptions!$C$14+T9*Assumptions!$D$14)*Assumptions!$B$5</f>
-        <v>1833</v>
+        <v>9275.66666666667</v>
       </c>
       <c r="U24" s="17" t="n">
         <f aca="false">(U7*Assumptions!$B$14+U8*Assumptions!$C$14+U9*Assumptions!$D$14)*Assumptions!$B$5</f>
-        <v>1833</v>
+        <v>9275.66666666667</v>
       </c>
       <c r="V24" s="17" t="n">
         <f aca="false">(V7*Assumptions!$B$14+V8*Assumptions!$C$14+V9*Assumptions!$D$14)*Assumptions!$B$5</f>
-        <v>1833</v>
+        <v>9275.66666666667</v>
       </c>
       <c r="W24" s="17" t="n">
         <f aca="false">(W7*Assumptions!$B$14+W8*Assumptions!$C$14+W9*Assumptions!$D$14)*Assumptions!$B$5</f>
@@ -6456,27 +6456,27 @@
       </c>
       <c r="Z24" s="17" t="n">
         <f aca="false">(Z7*Assumptions!$B$14+Z8*Assumptions!$C$14+Z9*Assumptions!$D$14)*Assumptions!$B$5</f>
-        <v>9275.66666666667</v>
+        <v>1833</v>
       </c>
       <c r="AA24" s="17" t="n">
         <f aca="false">(AA7*Assumptions!$B$14+AA8*Assumptions!$C$14+AA9*Assumptions!$D$14)*Assumptions!$B$5</f>
-        <v>9275.66666666667</v>
+        <v>1833</v>
       </c>
       <c r="AB24" s="17" t="n">
         <f aca="false">(AB7*Assumptions!$B$14+AB8*Assumptions!$C$14+AB9*Assumptions!$D$14)*Assumptions!$B$5</f>
-        <v>9275.66666666667</v>
+        <v>1833</v>
       </c>
       <c r="AC24" s="17" t="n">
         <f aca="false">(AC7*Assumptions!$B$14+AC8*Assumptions!$C$14+AC9*Assumptions!$D$14)*Assumptions!$B$5</f>
-        <v>1833</v>
+        <v>9275.66666666667</v>
       </c>
       <c r="AD24" s="17" t="n">
         <f aca="false">(AD7*Assumptions!$B$14+AD8*Assumptions!$C$14+AD9*Assumptions!$D$14)*Assumptions!$B$5</f>
-        <v>1833</v>
+        <v>9275.66666666667</v>
       </c>
       <c r="AE24" s="17" t="n">
         <f aca="false">(AE7*Assumptions!$B$14+AE8*Assumptions!$C$14+AE9*Assumptions!$D$14)*Assumptions!$B$5</f>
-        <v>1833</v>
+        <v>9275.66666666667</v>
       </c>
       <c r="AF24" s="17" t="n">
         <f aca="false">(AF7*Assumptions!$B$14+AF8*Assumptions!$C$14+AF9*Assumptions!$D$14)*Assumptions!$B$5</f>
@@ -6521,75 +6521,75 @@
       </c>
       <c r="E25" s="17" t="n">
         <f aca="false">E7*(Assumptions!$B$15*Assumptions!$B$23+Assumptions!$B$16)+E8*(Assumptions!$C$15*Assumptions!$B$23+Assumptions!$C$16)+E9*(Assumptions!$D$15*Assumptions!$B$23+Assumptions!$D$16)</f>
-        <v>0</v>
+        <v>133.333333333333</v>
       </c>
       <c r="F25" s="17" t="n">
         <f aca="false">F7*(Assumptions!$B$15*Assumptions!$B$23+Assumptions!$B$16)+F8*(Assumptions!$C$15*Assumptions!$B$23+Assumptions!$C$16)+F9*(Assumptions!$D$15*Assumptions!$B$23+Assumptions!$D$16)</f>
-        <v>0</v>
+        <v>133.333333333333</v>
       </c>
       <c r="G25" s="17" t="n">
         <f aca="false">G7*(Assumptions!$B$15*Assumptions!$B$23+Assumptions!$B$16)+G8*(Assumptions!$C$15*Assumptions!$B$23+Assumptions!$C$16)+G9*(Assumptions!$D$15*Assumptions!$B$23+Assumptions!$D$16)</f>
-        <v>0</v>
+        <v>133.333333333333</v>
       </c>
       <c r="H25" s="17" t="n">
         <f aca="false">H7*(Assumptions!$B$15*Assumptions!$B$23+Assumptions!$B$16)+H8*(Assumptions!$C$15*Assumptions!$B$23+Assumptions!$C$16)+H9*(Assumptions!$D$15*Assumptions!$B$23+Assumptions!$D$16)</f>
-        <v>133.333333333333</v>
+        <v>300</v>
       </c>
       <c r="I25" s="17" t="n">
         <f aca="false">I7*(Assumptions!$B$15*Assumptions!$B$23+Assumptions!$B$16)+I8*(Assumptions!$C$15*Assumptions!$B$23+Assumptions!$C$16)+I9*(Assumptions!$D$15*Assumptions!$B$23+Assumptions!$D$16)</f>
-        <v>133.333333333333</v>
+        <v>300</v>
       </c>
       <c r="J25" s="17" t="n">
         <f aca="false">J7*(Assumptions!$B$15*Assumptions!$B$23+Assumptions!$B$16)+J8*(Assumptions!$C$15*Assumptions!$B$23+Assumptions!$C$16)+J9*(Assumptions!$D$15*Assumptions!$B$23+Assumptions!$D$16)</f>
-        <v>133.333333333333</v>
+        <v>300</v>
       </c>
       <c r="K25" s="17" t="n">
         <f aca="false">K7*(Assumptions!$B$15*Assumptions!$B$23+Assumptions!$B$16)+K8*(Assumptions!$C$15*Assumptions!$B$23+Assumptions!$C$16)+K9*(Assumptions!$D$15*Assumptions!$B$23+Assumptions!$D$16)</f>
-        <v>300</v>
+        <v>133.333333333333</v>
       </c>
       <c r="L25" s="17" t="n">
         <f aca="false">L7*(Assumptions!$B$15*Assumptions!$B$23+Assumptions!$B$16)+L8*(Assumptions!$C$15*Assumptions!$B$23+Assumptions!$C$16)+L9*(Assumptions!$D$15*Assumptions!$B$23+Assumptions!$D$16)</f>
-        <v>300</v>
+        <v>133.333333333333</v>
       </c>
       <c r="M25" s="17" t="n">
         <f aca="false">M7*(Assumptions!$B$15*Assumptions!$B$23+Assumptions!$B$16)+M8*(Assumptions!$C$15*Assumptions!$B$23+Assumptions!$C$16)+M9*(Assumptions!$D$15*Assumptions!$B$23+Assumptions!$D$16)</f>
-        <v>300</v>
+        <v>133.333333333333</v>
       </c>
       <c r="N25" s="17" t="n">
         <f aca="false">N7*(Assumptions!$B$15*Assumptions!$B$23+Assumptions!$B$16)+N8*(Assumptions!$C$15*Assumptions!$B$23+Assumptions!$C$16)+N9*(Assumptions!$D$15*Assumptions!$B$23+Assumptions!$D$16)</f>
-        <v>133.333333333333</v>
+        <v>433.333333333333</v>
       </c>
       <c r="O25" s="17" t="n">
         <f aca="false">O7*(Assumptions!$B$15*Assumptions!$B$23+Assumptions!$B$16)+O8*(Assumptions!$C$15*Assumptions!$B$23+Assumptions!$C$16)+O9*(Assumptions!$D$15*Assumptions!$B$23+Assumptions!$D$16)</f>
-        <v>133.333333333333</v>
+        <v>433.333333333333</v>
       </c>
       <c r="P25" s="17" t="n">
         <f aca="false">P7*(Assumptions!$B$15*Assumptions!$B$23+Assumptions!$B$16)+P8*(Assumptions!$C$15*Assumptions!$B$23+Assumptions!$C$16)+P9*(Assumptions!$D$15*Assumptions!$B$23+Assumptions!$D$16)</f>
-        <v>133.333333333333</v>
+        <v>433.333333333333</v>
       </c>
       <c r="Q25" s="17" t="n">
         <f aca="false">Q7*(Assumptions!$B$15*Assumptions!$B$23+Assumptions!$B$16)+Q8*(Assumptions!$C$15*Assumptions!$B$23+Assumptions!$C$16)+Q9*(Assumptions!$D$15*Assumptions!$B$23+Assumptions!$D$16)</f>
-        <v>433.333333333333</v>
+        <v>133.333333333333</v>
       </c>
       <c r="R25" s="17" t="n">
         <f aca="false">R7*(Assumptions!$B$15*Assumptions!$B$23+Assumptions!$B$16)+R8*(Assumptions!$C$15*Assumptions!$B$23+Assumptions!$C$16)+R9*(Assumptions!$D$15*Assumptions!$B$23+Assumptions!$D$16)</f>
-        <v>433.333333333333</v>
+        <v>133.333333333333</v>
       </c>
       <c r="S25" s="17" t="n">
         <f aca="false">S7*(Assumptions!$B$15*Assumptions!$B$23+Assumptions!$B$16)+S8*(Assumptions!$C$15*Assumptions!$B$23+Assumptions!$C$16)+S9*(Assumptions!$D$15*Assumptions!$B$23+Assumptions!$D$16)</f>
-        <v>433.333333333333</v>
+        <v>133.333333333333</v>
       </c>
       <c r="T25" s="17" t="n">
         <f aca="false">T7*(Assumptions!$B$15*Assumptions!$B$23+Assumptions!$B$16)+T8*(Assumptions!$C$15*Assumptions!$B$23+Assumptions!$C$16)+T9*(Assumptions!$D$15*Assumptions!$B$23+Assumptions!$D$16)</f>
-        <v>133.333333333333</v>
+        <v>433.333333333333</v>
       </c>
       <c r="U25" s="17" t="n">
         <f aca="false">U7*(Assumptions!$B$15*Assumptions!$B$23+Assumptions!$B$16)+U8*(Assumptions!$C$15*Assumptions!$B$23+Assumptions!$C$16)+U9*(Assumptions!$D$15*Assumptions!$B$23+Assumptions!$D$16)</f>
-        <v>133.333333333333</v>
+        <v>433.333333333333</v>
       </c>
       <c r="V25" s="17" t="n">
         <f aca="false">V7*(Assumptions!$B$15*Assumptions!$B$23+Assumptions!$B$16)+V8*(Assumptions!$C$15*Assumptions!$B$23+Assumptions!$C$16)+V9*(Assumptions!$D$15*Assumptions!$B$23+Assumptions!$D$16)</f>
-        <v>133.333333333333</v>
+        <v>433.333333333333</v>
       </c>
       <c r="W25" s="17" t="n">
         <f aca="false">W7*(Assumptions!$B$15*Assumptions!$B$23+Assumptions!$B$16)+W8*(Assumptions!$C$15*Assumptions!$B$23+Assumptions!$C$16)+W9*(Assumptions!$D$15*Assumptions!$B$23+Assumptions!$D$16)</f>
@@ -6605,27 +6605,27 @@
       </c>
       <c r="Z25" s="17" t="n">
         <f aca="false">Z7*(Assumptions!$B$15*Assumptions!$B$23+Assumptions!$B$16)+Z8*(Assumptions!$C$15*Assumptions!$B$23+Assumptions!$C$16)+Z9*(Assumptions!$D$15*Assumptions!$B$23+Assumptions!$D$16)</f>
-        <v>433.333333333333</v>
+        <v>133.333333333333</v>
       </c>
       <c r="AA25" s="17" t="n">
         <f aca="false">AA7*(Assumptions!$B$15*Assumptions!$B$23+Assumptions!$B$16)+AA8*(Assumptions!$C$15*Assumptions!$B$23+Assumptions!$C$16)+AA9*(Assumptions!$D$15*Assumptions!$B$23+Assumptions!$D$16)</f>
-        <v>433.333333333333</v>
+        <v>133.333333333333</v>
       </c>
       <c r="AB25" s="17" t="n">
         <f aca="false">AB7*(Assumptions!$B$15*Assumptions!$B$23+Assumptions!$B$16)+AB8*(Assumptions!$C$15*Assumptions!$B$23+Assumptions!$C$16)+AB9*(Assumptions!$D$15*Assumptions!$B$23+Assumptions!$D$16)</f>
-        <v>433.333333333333</v>
+        <v>133.333333333333</v>
       </c>
       <c r="AC25" s="17" t="n">
         <f aca="false">AC7*(Assumptions!$B$15*Assumptions!$B$23+Assumptions!$B$16)+AC8*(Assumptions!$C$15*Assumptions!$B$23+Assumptions!$C$16)+AC9*(Assumptions!$D$15*Assumptions!$B$23+Assumptions!$D$16)</f>
-        <v>133.333333333333</v>
+        <v>433.333333333333</v>
       </c>
       <c r="AD25" s="17" t="n">
         <f aca="false">AD7*(Assumptions!$B$15*Assumptions!$B$23+Assumptions!$B$16)+AD8*(Assumptions!$C$15*Assumptions!$B$23+Assumptions!$C$16)+AD9*(Assumptions!$D$15*Assumptions!$B$23+Assumptions!$D$16)</f>
-        <v>133.333333333333</v>
+        <v>433.333333333333</v>
       </c>
       <c r="AE25" s="17" t="n">
         <f aca="false">AE7*(Assumptions!$B$15*Assumptions!$B$23+Assumptions!$B$16)+AE8*(Assumptions!$C$15*Assumptions!$B$23+Assumptions!$C$16)+AE9*(Assumptions!$D$15*Assumptions!$B$23+Assumptions!$D$16)</f>
-        <v>133.333333333333</v>
+        <v>433.333333333333</v>
       </c>
       <c r="AF25" s="17" t="n">
         <f aca="false">AF7*(Assumptions!$B$15*Assumptions!$B$23+Assumptions!$B$16)+AF8*(Assumptions!$C$15*Assumptions!$B$23+Assumptions!$C$16)+AF9*(Assumptions!$D$15*Assumptions!$B$23+Assumptions!$D$16)</f>
@@ -6670,135 +6670,135 @@
       </c>
       <c r="E26" s="17" t="n">
         <f aca="false">E12*(Assumptions!$B$17*Assumptions!$B$23+Assumptions!$B$18)+E13*(Assumptions!$C$17*Assumptions!$B$23+Assumptions!$C$18)+E14*(Assumptions!$D$17*Assumptions!$B$23+Assumptions!$D$18)</f>
-        <v>0</v>
+        <v>16.6666666666667</v>
       </c>
       <c r="F26" s="17" t="n">
         <f aca="false">F12*(Assumptions!$B$17*Assumptions!$B$23+Assumptions!$B$18)+F13*(Assumptions!$C$17*Assumptions!$B$23+Assumptions!$C$18)+F14*(Assumptions!$D$17*Assumptions!$B$23+Assumptions!$D$18)</f>
-        <v>0</v>
+        <v>33.1876398174217</v>
       </c>
       <c r="G26" s="17" t="n">
         <f aca="false">G12*(Assumptions!$B$17*Assumptions!$B$23+Assumptions!$B$18)+G13*(Assumptions!$C$17*Assumptions!$B$23+Assumptions!$C$18)+G14*(Assumptions!$D$17*Assumptions!$B$23+Assumptions!$D$18)</f>
-        <v>0</v>
+        <v>49.5641930482999</v>
       </c>
       <c r="H26" s="17" t="n">
         <f aca="false">H12*(Assumptions!$B$17*Assumptions!$B$23+Assumptions!$B$18)+H13*(Assumptions!$C$17*Assumptions!$B$23+Assumptions!$C$18)+H14*(Assumptions!$D$17*Assumptions!$B$23+Assumptions!$D$18)</f>
-        <v>16.6666666666667</v>
+        <v>82.4642554887215</v>
       </c>
       <c r="I26" s="17" t="n">
         <f aca="false">I12*(Assumptions!$B$17*Assumptions!$B$23+Assumptions!$B$18)+I13*(Assumptions!$C$17*Assumptions!$B$23+Assumptions!$C$18)+I14*(Assumptions!$D$17*Assumptions!$B$23+Assumptions!$D$18)</f>
-        <v>33.1876398174217</v>
+        <v>115.076718382904</v>
       </c>
       <c r="J26" s="17" t="n">
         <f aca="false">J12*(Assumptions!$B$17*Assumptions!$B$23+Assumptions!$B$18)+J13*(Assumptions!$C$17*Assumptions!$B$23+Assumptions!$C$18)+J14*(Assumptions!$D$17*Assumptions!$B$23+Assumptions!$D$18)</f>
-        <v>49.5641930482999</v>
+        <v>147.404095814191</v>
       </c>
       <c r="K26" s="17" t="n">
         <f aca="false">K12*(Assumptions!$B$17*Assumptions!$B$23+Assumptions!$B$18)+K13*(Assumptions!$C$17*Assumptions!$B$23+Assumptions!$C$18)+K14*(Assumptions!$D$17*Assumptions!$B$23+Assumptions!$D$18)</f>
-        <v>82.4642554887215</v>
+        <v>162.782213222121</v>
       </c>
       <c r="L26" s="17" t="n">
         <f aca="false">L12*(Assumptions!$B$17*Assumptions!$B$23+Assumptions!$B$18)+L13*(Assumptions!$C$17*Assumptions!$B$23+Assumptions!$C$18)+L14*(Assumptions!$D$17*Assumptions!$B$23+Assumptions!$D$18)</f>
-        <v>115.076718382904</v>
+        <v>178.025901110455</v>
       </c>
       <c r="M26" s="17" t="n">
         <f aca="false">M12*(Assumptions!$B$17*Assumptions!$B$23+Assumptions!$B$18)+M13*(Assumptions!$C$17*Assumptions!$B$23+Assumptions!$C$18)+M14*(Assumptions!$D$17*Assumptions!$B$23+Assumptions!$D$18)</f>
-        <v>147.404095814191</v>
+        <v>193.136334609755</v>
       </c>
       <c r="N26" s="17" t="n">
         <f aca="false">N12*(Assumptions!$B$17*Assumptions!$B$23+Assumptions!$B$18)+N13*(Assumptions!$C$17*Assumptions!$B$23+Assumptions!$C$18)+N14*(Assumptions!$D$17*Assumptions!$B$23+Assumptions!$D$18)</f>
-        <v>162.782213222121</v>
+        <v>241.44801191138</v>
       </c>
       <c r="O26" s="17" t="n">
         <f aca="false">O12*(Assumptions!$B$17*Assumptions!$B$23+Assumptions!$B$18)+O13*(Assumptions!$C$17*Assumptions!$B$23+Assumptions!$C$18)+O14*(Assumptions!$D$17*Assumptions!$B$23+Assumptions!$D$18)</f>
-        <v>178.025901110455</v>
+        <v>289.337367325466</v>
       </c>
       <c r="P26" s="17" t="n">
         <f aca="false">P12*(Assumptions!$B$17*Assumptions!$B$23+Assumptions!$B$18)+P13*(Assumptions!$C$17*Assumptions!$B$23+Assumptions!$C$18)+P14*(Assumptions!$D$17*Assumptions!$B$23+Assumptions!$D$18)</f>
-        <v>193.136334609755</v>
+        <v>336.808092625651</v>
       </c>
       <c r="Q26" s="17" t="n">
         <f aca="false">Q12*(Assumptions!$B$17*Assumptions!$B$23+Assumptions!$B$18)+Q13*(Assumptions!$C$17*Assumptions!$B$23+Assumptions!$C$18)+Q14*(Assumptions!$D$17*Assumptions!$B$23+Assumptions!$D$18)</f>
-        <v>241.44801191138</v>
+        <v>350.53051398019</v>
       </c>
       <c r="R26" s="17" t="n">
         <f aca="false">R12*(Assumptions!$B$17*Assumptions!$B$23+Assumptions!$B$18)+R13*(Assumptions!$C$17*Assumptions!$B$23+Assumptions!$C$18)+R14*(Assumptions!$D$17*Assumptions!$B$23+Assumptions!$D$18)</f>
-        <v>289.337367325466</v>
+        <v>364.132979265892</v>
       </c>
       <c r="S26" s="17" t="n">
         <f aca="false">S12*(Assumptions!$B$17*Assumptions!$B$23+Assumptions!$B$18)+S13*(Assumptions!$C$17*Assumptions!$B$23+Assumptions!$C$18)+S14*(Assumptions!$D$17*Assumptions!$B$23+Assumptions!$D$18)</f>
-        <v>336.808092625651</v>
+        <v>377.616537092042</v>
       </c>
       <c r="T26" s="17" t="n">
         <f aca="false">T12*(Assumptions!$B$17*Assumptions!$B$23+Assumptions!$B$18)+T13*(Assumptions!$C$17*Assumptions!$B$23+Assumptions!$C$18)+T14*(Assumptions!$D$17*Assumptions!$B$23+Assumptions!$D$18)</f>
-        <v>350.53051398019</v>
+        <v>424.315560234724</v>
       </c>
       <c r="U26" s="17" t="n">
         <f aca="false">U12*(Assumptions!$B$17*Assumptions!$B$23+Assumptions!$B$18)+U13*(Assumptions!$C$17*Assumptions!$B$23+Assumptions!$C$18)+U14*(Assumptions!$D$17*Assumptions!$B$23+Assumptions!$D$18)</f>
-        <v>364.132979265892</v>
+        <v>470.606358685127</v>
       </c>
       <c r="V26" s="17" t="n">
         <f aca="false">V12*(Assumptions!$B$17*Assumptions!$B$23+Assumptions!$B$18)+V13*(Assumptions!$C$17*Assumptions!$B$23+Assumptions!$C$18)+V14*(Assumptions!$D$17*Assumptions!$B$23+Assumptions!$D$18)</f>
-        <v>377.616537092042</v>
+        <v>516.492500984696</v>
       </c>
       <c r="W26" s="17" t="n">
         <f aca="false">W12*(Assumptions!$B$17*Assumptions!$B$23+Assumptions!$B$18)+W13*(Assumptions!$C$17*Assumptions!$B$23+Assumptions!$C$18)+W14*(Assumptions!$D$17*Assumptions!$B$23+Assumptions!$D$18)</f>
-        <v>424.315560234724</v>
+        <v>561.977524480069</v>
       </c>
       <c r="X26" s="17" t="n">
         <f aca="false">X12*(Assumptions!$B$17*Assumptions!$B$23+Assumptions!$B$18)+X13*(Assumptions!$C$17*Assumptions!$B$23+Assumptions!$C$18)+X14*(Assumptions!$D$17*Assumptions!$B$23+Assumptions!$D$18)</f>
-        <v>470.606358685127</v>
+        <v>607.064935595781</v>
       </c>
       <c r="Y26" s="17" t="n">
         <f aca="false">Y12*(Assumptions!$B$17*Assumptions!$B$23+Assumptions!$B$18)+Y13*(Assumptions!$C$17*Assumptions!$B$23+Assumptions!$C$18)+Y14*(Assumptions!$D$17*Assumptions!$B$23+Assumptions!$D$18)</f>
-        <v>516.492500984696</v>
+        <v>651.758210104564</v>
       </c>
       <c r="Z26" s="17" t="n">
         <f aca="false">Z12*(Assumptions!$B$17*Assumptions!$B$23+Assumptions!$B$18)+Z13*(Assumptions!$C$17*Assumptions!$B$23+Assumptions!$C$18)+Z14*(Assumptions!$D$17*Assumptions!$B$23+Assumptions!$D$18)</f>
-        <v>561.977524480069</v>
+        <v>662.727460061968</v>
       </c>
       <c r="AA26" s="17" t="n">
         <f aca="false">AA12*(Assumptions!$B$17*Assumptions!$B$23+Assumptions!$B$18)+AA13*(Assumptions!$C$17*Assumptions!$B$23+Assumptions!$C$18)+AA14*(Assumptions!$D$17*Assumptions!$B$23+Assumptions!$D$18)</f>
-        <v>607.064935595781</v>
+        <v>673.600821103778</v>
       </c>
       <c r="AB26" s="17" t="n">
         <f aca="false">AB12*(Assumptions!$B$17*Assumptions!$B$23+Assumptions!$B$18)+AB13*(Assumptions!$C$17*Assumptions!$B$23+Assumptions!$C$18)+AB14*(Assumptions!$D$17*Assumptions!$B$23+Assumptions!$D$18)</f>
-        <v>651.758210104564</v>
+        <v>684.379131453591</v>
       </c>
       <c r="AC26" s="17" t="n">
         <f aca="false">AC12*(Assumptions!$B$17*Assumptions!$B$23+Assumptions!$B$18)+AC13*(Assumptions!$C$17*Assumptions!$B$23+Assumptions!$C$18)+AC14*(Assumptions!$D$17*Assumptions!$B$23+Assumptions!$D$18)</f>
-        <v>662.727460061968</v>
+        <v>728.396555340911</v>
       </c>
       <c r="AD26" s="17" t="n">
         <f aca="false">AD12*(Assumptions!$B$17*Assumptions!$B$23+Assumptions!$B$18)+AD13*(Assumptions!$C$17*Assumptions!$B$23+Assumptions!$C$18)+AD14*(Assumptions!$D$17*Assumptions!$B$23+Assumptions!$D$18)</f>
-        <v>673.600821103778</v>
+        <v>772.029196033379</v>
       </c>
       <c r="AE26" s="17" t="n">
         <f aca="false">AE12*(Assumptions!$B$17*Assumptions!$B$23+Assumptions!$B$18)+AE13*(Assumptions!$C$17*Assumptions!$B$23+Assumptions!$C$18)+AE14*(Assumptions!$D$17*Assumptions!$B$23+Assumptions!$D$18)</f>
-        <v>684.379131453591</v>
+        <v>815.280417155988</v>
       </c>
       <c r="AF26" s="17" t="n">
         <f aca="false">AF12*(Assumptions!$B$17*Assumptions!$B$23+Assumptions!$B$18)+AF13*(Assumptions!$C$17*Assumptions!$B$23+Assumptions!$C$18)+AF14*(Assumptions!$D$17*Assumptions!$B$23+Assumptions!$D$18)</f>
-        <v>728.396555340911</v>
+        <v>858.153552930228</v>
       </c>
       <c r="AG26" s="17" t="n">
         <f aca="false">AG12*(Assumptions!$B$17*Assumptions!$B$23+Assumptions!$B$18)+AG13*(Assumptions!$C$17*Assumptions!$B$23+Assumptions!$C$18)+AG14*(Assumptions!$D$17*Assumptions!$B$23+Assumptions!$D$18)</f>
-        <v>772.029196033379</v>
+        <v>900.651908431121</v>
       </c>
       <c r="AH26" s="17" t="n">
         <f aca="false">AH12*(Assumptions!$B$17*Assumptions!$B$23+Assumptions!$B$18)+AH13*(Assumptions!$C$17*Assumptions!$B$23+Assumptions!$C$18)+AH14*(Assumptions!$D$17*Assumptions!$B$23+Assumptions!$D$18)</f>
-        <v>815.280417155988</v>
+        <v>942.778759842011</v>
       </c>
       <c r="AI26" s="17" t="n">
         <f aca="false">AI12*(Assumptions!$B$17*Assumptions!$B$23+Assumptions!$B$18)+AI13*(Assumptions!$C$17*Assumptions!$B$23+Assumptions!$C$18)+AI14*(Assumptions!$D$17*Assumptions!$B$23+Assumptions!$D$18)</f>
-        <v>858.153552930228</v>
+        <v>984.53735470712</v>
       </c>
       <c r="AJ26" s="17" t="n">
         <f aca="false">AJ12*(Assumptions!$B$17*Assumptions!$B$23+Assumptions!$B$18)+AJ13*(Assumptions!$C$17*Assumptions!$B$23+Assumptions!$C$18)+AJ14*(Assumptions!$D$17*Assumptions!$B$23+Assumptions!$D$18)</f>
-        <v>900.651908431121</v>
+        <v>1025.9309121819</v>
       </c>
       <c r="AK26" s="17" t="n">
         <f aca="false">AK12*(Assumptions!$B$17*Assumptions!$B$23+Assumptions!$B$18)+AK13*(Assumptions!$C$17*Assumptions!$B$23+Assumptions!$C$18)+AK14*(Assumptions!$D$17*Assumptions!$B$23+Assumptions!$D$18)</f>
-        <v>942.778759842011</v>
+        <v>1066.96262328121</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6819,135 +6819,135 @@
       </c>
       <c r="E27" s="12" t="n">
         <f aca="false">SUM(E24:E26)</f>
-        <v>0</v>
+        <v>1983</v>
       </c>
       <c r="F27" s="12" t="n">
         <f aca="false">SUM(F24:F26)</f>
-        <v>0</v>
+        <v>1999.52097315076</v>
       </c>
       <c r="G27" s="12" t="n">
         <f aca="false">SUM(G24:G26)</f>
-        <v>0</v>
+        <v>2015.89752638163</v>
       </c>
       <c r="H27" s="12" t="n">
         <f aca="false">SUM(H24:H26)</f>
-        <v>1983</v>
+        <v>7825.13092215539</v>
       </c>
       <c r="I27" s="12" t="n">
         <f aca="false">SUM(I24:I26)</f>
-        <v>1999.52097315076</v>
+        <v>7857.74338504957</v>
       </c>
       <c r="J27" s="12" t="n">
         <f aca="false">SUM(J24:J26)</f>
-        <v>2015.89752638163</v>
+        <v>7890.07076248086</v>
       </c>
       <c r="K27" s="12" t="n">
         <f aca="false">SUM(K24:K26)</f>
-        <v>7825.13092215539</v>
+        <v>2129.11554655545</v>
       </c>
       <c r="L27" s="12" t="n">
         <f aca="false">SUM(L24:L26)</f>
-        <v>7857.74338504957</v>
+        <v>2144.35923444379</v>
       </c>
       <c r="M27" s="12" t="n">
         <f aca="false">SUM(M24:M26)</f>
-        <v>7890.07076248086</v>
+        <v>2159.46966794309</v>
       </c>
       <c r="N27" s="12" t="n">
         <f aca="false">SUM(N24:N26)</f>
-        <v>2129.11554655545</v>
+        <v>9950.44801191138</v>
       </c>
       <c r="O27" s="12" t="n">
         <f aca="false">SUM(O24:O26)</f>
-        <v>2144.35923444379</v>
+        <v>9998.33736732547</v>
       </c>
       <c r="P27" s="12" t="n">
         <f aca="false">SUM(P24:P26)</f>
-        <v>2159.46966794309</v>
+        <v>10045.8080926257</v>
       </c>
       <c r="Q27" s="12" t="n">
         <f aca="false">SUM(Q24:Q26)</f>
-        <v>9950.44801191138</v>
+        <v>2316.86384731352</v>
       </c>
       <c r="R27" s="12" t="n">
         <f aca="false">SUM(R24:R26)</f>
-        <v>9998.33736732547</v>
+        <v>2330.46631259923</v>
       </c>
       <c r="S27" s="12" t="n">
         <f aca="false">SUM(S24:S26)</f>
-        <v>10045.8080926257</v>
+        <v>2343.94987042538</v>
       </c>
       <c r="T27" s="12" t="n">
         <f aca="false">SUM(T24:T26)</f>
-        <v>2316.86384731352</v>
+        <v>10133.3155602347</v>
       </c>
       <c r="U27" s="12" t="n">
         <f aca="false">SUM(U24:U26)</f>
-        <v>2330.46631259923</v>
+        <v>10179.6063586851</v>
       </c>
       <c r="V27" s="12" t="n">
         <f aca="false">SUM(V24:V26)</f>
-        <v>2343.94987042538</v>
+        <v>10225.4925009847</v>
       </c>
       <c r="W27" s="12" t="n">
         <f aca="false">SUM(W24:W26)</f>
-        <v>10133.3155602347</v>
+        <v>10270.9775244801</v>
       </c>
       <c r="X27" s="12" t="n">
         <f aca="false">SUM(X24:X26)</f>
-        <v>10179.6063586851</v>
+        <v>10316.0649355958</v>
       </c>
       <c r="Y27" s="12" t="n">
         <f aca="false">SUM(Y24:Y26)</f>
-        <v>10225.4925009847</v>
+        <v>10360.7582101046</v>
       </c>
       <c r="Z27" s="12" t="n">
         <f aca="false">SUM(Z24:Z26)</f>
-        <v>10270.9775244801</v>
+        <v>2629.0607933953</v>
       </c>
       <c r="AA27" s="12" t="n">
         <f aca="false">SUM(AA24:AA26)</f>
-        <v>10316.0649355958</v>
+        <v>2639.93415443711</v>
       </c>
       <c r="AB27" s="12" t="n">
         <f aca="false">SUM(AB24:AB26)</f>
-        <v>10360.7582101046</v>
+        <v>2650.71246478692</v>
       </c>
       <c r="AC27" s="12" t="n">
         <f aca="false">SUM(AC24:AC26)</f>
-        <v>2629.0607933953</v>
+        <v>10437.3965553409</v>
       </c>
       <c r="AD27" s="12" t="n">
         <f aca="false">SUM(AD24:AD26)</f>
-        <v>2639.93415443711</v>
+        <v>10481.0291960334</v>
       </c>
       <c r="AE27" s="12" t="n">
         <f aca="false">SUM(AE24:AE26)</f>
-        <v>2650.71246478692</v>
+        <v>10524.280417156</v>
       </c>
       <c r="AF27" s="12" t="n">
         <f aca="false">SUM(AF24:AF26)</f>
-        <v>10437.3965553409</v>
+        <v>10567.1535529302</v>
       </c>
       <c r="AG27" s="12" t="n">
         <f aca="false">SUM(AG24:AG26)</f>
-        <v>10481.0291960334</v>
+        <v>10609.6519084311</v>
       </c>
       <c r="AH27" s="12" t="n">
         <f aca="false">SUM(AH24:AH26)</f>
-        <v>10524.280417156</v>
+        <v>10651.778759842</v>
       </c>
       <c r="AI27" s="12" t="n">
         <f aca="false">SUM(AI24:AI26)</f>
-        <v>10567.1535529302</v>
+        <v>10693.5373547071</v>
       </c>
       <c r="AJ27" s="12" t="n">
         <f aca="false">SUM(AJ24:AJ26)</f>
-        <v>10609.6519084311</v>
+        <v>10734.9309121819</v>
       </c>
       <c r="AK27" s="12" t="n">
         <f aca="false">SUM(AK24:AK26)</f>
-        <v>10651.778759842</v>
+        <v>10775.9626232812</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6968,135 +6968,135 @@
       </c>
       <c r="E28" s="12" t="n">
         <f aca="false">E21-E27</f>
-        <v>0</v>
+        <v>1874.95</v>
       </c>
       <c r="F28" s="12" t="n">
         <f aca="false">F21-F27</f>
-        <v>0</v>
+        <v>2106.24362411057</v>
       </c>
       <c r="G28" s="12" t="n">
         <f aca="false">G21-G27</f>
-        <v>0</v>
+        <v>2335.51536934287</v>
       </c>
       <c r="H28" s="12" t="n">
         <f aca="false">H21-H27</f>
-        <v>1874.95</v>
+        <v>6137.56624350877</v>
       </c>
       <c r="I28" s="12" t="n">
         <f aca="false">I21-I27</f>
-        <v>2106.24362411057</v>
+        <v>6759.35045553487</v>
       </c>
       <c r="J28" s="12" t="n">
         <f aca="false">J21-J27</f>
-        <v>2335.51536934287</v>
+        <v>7375.69927188167</v>
       </c>
       <c r="K28" s="12" t="n">
         <f aca="false">K21-K27</f>
-        <v>6137.56624350877</v>
+        <v>4411.87687333024</v>
       </c>
       <c r="L28" s="12" t="n">
         <f aca="false">L21-L27</f>
-        <v>6759.35045553487</v>
+        <v>4620.99366969364</v>
       </c>
       <c r="M28" s="12" t="n">
         <f aca="false">M21-M27</f>
-        <v>7375.69927188167</v>
+        <v>4828.28244837914</v>
       </c>
       <c r="N28" s="12" t="n">
         <f aca="false">N21-N27</f>
-        <v>7344.91929321593</v>
+        <v>14750.4163903236</v>
       </c>
       <c r="O28" s="12" t="n">
         <f aca="false">O21-O27</f>
-        <v>7778.39657383107</v>
+        <v>16461.2607913919</v>
       </c>
       <c r="P28" s="12" t="n">
         <f aca="false">P21-P27</f>
-        <v>8208.08456470137</v>
+        <v>18157.149656302</v>
       </c>
       <c r="Q28" s="12" t="n">
         <f aca="false">Q21-Q27</f>
-        <v>14750.4163903236</v>
+        <v>13721.8137205327</v>
       </c>
       <c r="R28" s="12" t="n">
         <f aca="false">R21-R27</f>
-        <v>16461.2607913919</v>
+        <v>14099.5466709651</v>
       </c>
       <c r="S28" s="12" t="n">
         <f aca="false">S21-S27</f>
-        <v>18157.149656302</v>
+        <v>14473.9776269</v>
       </c>
       <c r="T28" s="12" t="n">
         <f aca="false">T21-T27</f>
-        <v>13721.8137205327</v>
+        <v>20961.5354530887</v>
       </c>
       <c r="U28" s="12" t="n">
         <f aca="false">U21-U27</f>
-        <v>14099.5466709651</v>
+        <v>22618.084667717</v>
       </c>
       <c r="V28" s="12" t="n">
         <f aca="false">V21-V27</f>
-        <v>14473.9776269</v>
+        <v>24260.1529735837</v>
       </c>
       <c r="W28" s="12" t="n">
         <f aca="false">W21-W27</f>
-        <v>20961.5354530887</v>
+        <v>25887.8669571595</v>
       </c>
       <c r="X28" s="12" t="n">
         <f aca="false">X21-X27</f>
-        <v>22618.084667717</v>
+        <v>27501.3520983453</v>
       </c>
       <c r="Y28" s="12" t="n">
         <f aca="false">Y21-Y27</f>
-        <v>24260.1529735837</v>
+        <v>29100.7327801458</v>
       </c>
       <c r="Z28" s="12" t="n">
         <f aca="false">Z21-Z27</f>
-        <v>25887.8669571595</v>
+        <v>24569.7322982574</v>
       </c>
       <c r="AA28" s="12" t="n">
         <f aca="false">AA21-AA27</f>
-        <v>27501.3520983453</v>
+        <v>24852.6369648151</v>
       </c>
       <c r="AB28" s="12" t="n">
         <f aca="false">AB21-AB27</f>
-        <v>29100.7327801458</v>
+        <v>25133.0685888404</v>
       </c>
       <c r="AC28" s="12" t="n">
         <f aca="false">AC21-AC27</f>
-        <v>24569.7322982574</v>
+        <v>31527.4487887092</v>
       </c>
       <c r="AD28" s="12" t="n">
         <f aca="false">AD21-AD27</f>
-        <v>24852.6369648151</v>
+        <v>33091.6348995764</v>
       </c>
       <c r="AE28" s="12" t="n">
         <f aca="false">AE21-AE27</f>
-        <v>25133.0685888404</v>
+        <v>34642.1475040017</v>
       </c>
       <c r="AF28" s="12" t="n">
         <f aca="false">AF21-AF27</f>
-        <v>31527.4487887092</v>
+        <v>36179.1061304588</v>
       </c>
       <c r="AG28" s="12" t="n">
         <f aca="false">AG21-AG27</f>
-        <v>33091.6348995764</v>
+        <v>37702.6292625499</v>
       </c>
       <c r="AH28" s="12" t="n">
         <f aca="false">AH21-AH27</f>
-        <v>34642.1475040017</v>
+        <v>39212.8343481398</v>
       </c>
       <c r="AI28" s="12" t="n">
         <f aca="false">AI21-AI27</f>
-        <v>36179.1061304588</v>
+        <v>40709.8378084097</v>
       </c>
       <c r="AJ28" s="12" t="n">
         <f aca="false">AJ21-AJ27</f>
-        <v>37702.6292625499</v>
+        <v>42193.7550468321</v>
       </c>
       <c r="AK28" s="12" t="n">
         <f aca="false">AK21-AK27</f>
-        <v>39212.8343481398</v>
+        <v>43664.7004580672</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7117,135 +7117,135 @@
       </c>
       <c r="E29" s="13" t="n">
         <f aca="false">IF(E21=0,0,E28/E21)</f>
-        <v>0</v>
+        <v>0.485996448891251</v>
       </c>
       <c r="F29" s="13" t="n">
         <f aca="false">IF(F21=0,0,F28/F21)</f>
-        <v>0</v>
+        <v>0.512996684104954</v>
       </c>
       <c r="G29" s="13" t="n">
         <f aca="false">IF(G21=0,0,G28/G21)</f>
-        <v>0</v>
+        <v>0.536725754441193</v>
       </c>
       <c r="H29" s="13" t="n">
         <f aca="false">IF(H21=0,0,H28/H21)</f>
-        <v>0.485996448891251</v>
+        <v>0.439568814727411</v>
       </c>
       <c r="I29" s="13" t="n">
         <f aca="false">IF(I21=0,0,I28/I21)</f>
-        <v>0.512996684104954</v>
+        <v>0.462427793736091</v>
       </c>
       <c r="J29" s="13" t="n">
         <f aca="false">IF(J21=0,0,J28/J21)</f>
-        <v>0.536725754441193</v>
+        <v>0.483152782681733</v>
       </c>
       <c r="K29" s="13" t="n">
         <f aca="false">IF(K21=0,0,K28/K21)</f>
-        <v>0.439568814727411</v>
+        <v>0.674496558032602</v>
       </c>
       <c r="L29" s="13" t="n">
         <f aca="false">IF(L21=0,0,L28/L21)</f>
-        <v>0.462427793736091</v>
+        <v>0.683038081704152</v>
       </c>
       <c r="M29" s="13" t="n">
         <f aca="false">IF(M21=0,0,M28/M21)</f>
-        <v>0.483152782681733</v>
+        <v>0.690963612905082</v>
       </c>
       <c r="N29" s="13" t="n">
         <f aca="false">IF(N21=0,0,N28/N21)</f>
-        <v>0.775268343154327</v>
+        <v>0.597161951505995</v>
       </c>
       <c r="O29" s="13" t="n">
         <f aca="false">IF(O21=0,0,O28/O21)</f>
-        <v>0.783894789322987</v>
+        <v>0.622128147700859</v>
       </c>
       <c r="P29" s="13" t="n">
         <f aca="false">IF(P21=0,0,P28/P21)</f>
-        <v>0.79170886213997</v>
+        <v>0.643803030091494</v>
       </c>
       <c r="Q29" s="13" t="n">
         <f aca="false">IF(Q21=0,0,Q28/Q21)</f>
-        <v>0.597161951505995</v>
+        <v>0.855545207046353</v>
       </c>
       <c r="R29" s="13" t="n">
         <f aca="false">IF(R21=0,0,R28/R21)</f>
-        <v>0.622128147700859</v>
+        <v>0.858157974985747</v>
       </c>
       <c r="S29" s="13" t="n">
         <f aca="false">IF(S21=0,0,S28/S21)</f>
-        <v>0.643803030091494</v>
+        <v>0.860627900150114</v>
       </c>
       <c r="T29" s="13" t="n">
         <f aca="false">IF(T21=0,0,T28/T21)</f>
-        <v>0.855545207046353</v>
+        <v>0.674115963575679</v>
       </c>
       <c r="U29" s="13" t="n">
         <f aca="false">IF(U21=0,0,U28/U21)</f>
-        <v>0.858157974985747</v>
+        <v>0.689624298537036</v>
       </c>
       <c r="V29" s="13" t="n">
         <f aca="false">IF(V21=0,0,V28/V21)</f>
-        <v>0.860627900150114</v>
+        <v>0.703485541294985</v>
       </c>
       <c r="W29" s="13" t="n">
         <f aca="false">IF(W21=0,0,W28/W21)</f>
-        <v>0.674115963575679</v>
+        <v>0.715948402895027</v>
       </c>
       <c r="X29" s="13" t="n">
         <f aca="false">IF(X21=0,0,X28/X21)</f>
-        <v>0.689624298537036</v>
+        <v>0.727213920338951</v>
       </c>
       <c r="Y29" s="13" t="n">
         <f aca="false">IF(Y21=0,0,Y28/Y21)</f>
-        <v>0.703485541294985</v>
+        <v>0.737446357192525</v>
       </c>
       <c r="Z29" s="13" t="n">
         <f aca="false">IF(Z21=0,0,Z28/Z21)</f>
-        <v>0.715948402895027</v>
+        <v>0.903339064180677</v>
       </c>
       <c r="AA29" s="13" t="n">
         <f aca="false">IF(AA21=0,0,AA28/AA21)</f>
-        <v>0.727213920338951</v>
+        <v>0.903976454476153</v>
       </c>
       <c r="AB29" s="13" t="n">
         <f aca="false">IF(AB21=0,0,AB28/AB21)</f>
-        <v>0.737446357192525</v>
+        <v>0.904594970005321</v>
       </c>
       <c r="AC29" s="13" t="n">
         <f aca="false">IF(AC21=0,0,AC28/AC21)</f>
-        <v>0.903339064180677</v>
+        <v>0.751282377671844</v>
       </c>
       <c r="AD29" s="13" t="n">
         <f aca="false">IF(AD21=0,0,AD28/AD21)</f>
-        <v>0.903976454476153</v>
+        <v>0.759458609805559</v>
       </c>
       <c r="AE29" s="13" t="n">
         <f aca="false">IF(AE21=0,0,AE28/AE21)</f>
-        <v>0.904594970005321</v>
+        <v>0.766988869796675</v>
       </c>
       <c r="AF29" s="13" t="n">
         <f aca="false">IF(AF21=0,0,AF28/AF21)</f>
-        <v>0.751282377671844</v>
+        <v>0.773946544076441</v>
       </c>
       <c r="AG29" s="13" t="n">
         <f aca="false">IF(AG21=0,0,AG28/AG21)</f>
-        <v>0.759458609805559</v>
+        <v>0.780394308625529</v>
       </c>
       <c r="AH29" s="13" t="n">
         <f aca="false">IF(AH21=0,0,AH28/AH21)</f>
-        <v>0.766988869796675</v>
+        <v>0.78638601413039</v>
       </c>
       <c r="AI29" s="13" t="n">
         <f aca="false">IF(AI21=0,0,AI28/AI21)</f>
-        <v>0.773946544076441</v>
+        <v>0.791968186509667</v>
       </c>
       <c r="AJ29" s="13" t="n">
         <f aca="false">IF(AJ21=0,0,AJ28/AJ21)</f>
-        <v>0.780394308625529</v>
+        <v>0.797181231355439</v>
       </c>
       <c r="AK29" s="13" t="n">
         <f aca="false">IF(AK21=0,0,AK28/AK21)</f>
-        <v>0.78638601413039</v>
+        <v>0.802060408280128</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8612,135 +8612,135 @@
       </c>
       <c r="E42" s="33" t="n">
         <f aca="false">E28-E40</f>
-        <v>-2658.33333333333</v>
+        <v>-783.383333333333</v>
       </c>
       <c r="F42" s="33" t="n">
         <f aca="false">F28-F40</f>
-        <v>-2658.33333333333</v>
+        <v>-552.089709222762</v>
       </c>
       <c r="G42" s="33" t="n">
         <f aca="false">G28-G40</f>
-        <v>-2658.33333333333</v>
+        <v>-322.817963990467</v>
       </c>
       <c r="H42" s="33" t="n">
         <f aca="false">H28-H40</f>
-        <v>-783.383333333333</v>
+        <v>3479.23291017543</v>
       </c>
       <c r="I42" s="33" t="n">
         <f aca="false">I28-I40</f>
-        <v>-552.089709222762</v>
+        <v>4101.01712220154</v>
       </c>
       <c r="J42" s="33" t="n">
         <f aca="false">J28-J40</f>
-        <v>-322.817963990467</v>
+        <v>4717.36593854833</v>
       </c>
       <c r="K42" s="33" t="n">
         <f aca="false">K28-K40</f>
-        <v>3479.23291017543</v>
+        <v>1753.5435399969</v>
       </c>
       <c r="L42" s="33" t="n">
         <f aca="false">L28-L40</f>
-        <v>4101.01712220154</v>
+        <v>1962.66033636031</v>
       </c>
       <c r="M42" s="33" t="n">
         <f aca="false">M28-M40</f>
-        <v>4717.36593854833</v>
+        <v>2169.94911504581</v>
       </c>
       <c r="N42" s="33" t="n">
         <f aca="false">N28-N40</f>
-        <v>3769.91929321593</v>
+        <v>11175.4163903236</v>
       </c>
       <c r="O42" s="33" t="n">
         <f aca="false">O28-O40</f>
-        <v>4203.39657383107</v>
+        <v>12886.2607913919</v>
       </c>
       <c r="P42" s="33" t="n">
         <f aca="false">P28-P40</f>
-        <v>4633.08456470137</v>
+        <v>14582.149656302</v>
       </c>
       <c r="Q42" s="33" t="n">
         <f aca="false">Q28-Q40</f>
-        <v>11175.4163903236</v>
+        <v>10146.8137205327</v>
       </c>
       <c r="R42" s="33" t="n">
         <f aca="false">R28-R40</f>
-        <v>12886.2607913919</v>
+        <v>10524.5466709651</v>
       </c>
       <c r="S42" s="33" t="n">
         <f aca="false">S28-S40</f>
-        <v>14582.149656302</v>
+        <v>10898.9776269</v>
       </c>
       <c r="T42" s="33" t="n">
         <f aca="false">T28-T40</f>
-        <v>10146.8137205327</v>
+        <v>17386.5354530887</v>
       </c>
       <c r="U42" s="33" t="n">
         <f aca="false">U28-U40</f>
-        <v>10524.5466709651</v>
+        <v>19043.084667717</v>
       </c>
       <c r="V42" s="33" t="n">
         <f aca="false">V28-V40</f>
-        <v>10898.9776269</v>
+        <v>20685.1529735837</v>
       </c>
       <c r="W42" s="33" t="n">
         <f aca="false">W28-W40</f>
-        <v>17386.5354530887</v>
+        <v>22312.8669571595</v>
       </c>
       <c r="X42" s="33" t="n">
         <f aca="false">X28-X40</f>
-        <v>19043.084667717</v>
+        <v>23926.3520983453</v>
       </c>
       <c r="Y42" s="33" t="n">
         <f aca="false">Y28-Y40</f>
-        <v>20685.1529735837</v>
+        <v>25525.7327801458</v>
       </c>
       <c r="Z42" s="33" t="n">
         <f aca="false">Z28-Z40</f>
-        <v>21487.8669571595</v>
+        <v>20169.7322982574</v>
       </c>
       <c r="AA42" s="33" t="n">
         <f aca="false">AA28-AA40</f>
-        <v>23101.3520983453</v>
+        <v>20452.6369648151</v>
       </c>
       <c r="AB42" s="33" t="n">
         <f aca="false">AB28-AB40</f>
-        <v>24700.7327801458</v>
+        <v>20733.0685888404</v>
       </c>
       <c r="AC42" s="33" t="n">
         <f aca="false">AC28-AC40</f>
-        <v>20169.7322982574</v>
+        <v>27127.4487887092</v>
       </c>
       <c r="AD42" s="33" t="n">
         <f aca="false">AD28-AD40</f>
-        <v>20452.6369648151</v>
+        <v>28691.6348995764</v>
       </c>
       <c r="AE42" s="33" t="n">
         <f aca="false">AE28-AE40</f>
-        <v>20733.0685888404</v>
+        <v>30242.1475040017</v>
       </c>
       <c r="AF42" s="33" t="n">
         <f aca="false">AF28-AF40</f>
-        <v>27127.4487887092</v>
+        <v>31779.1061304588</v>
       </c>
       <c r="AG42" s="33" t="n">
         <f aca="false">AG28-AG40</f>
-        <v>28691.6348995764</v>
+        <v>33302.6292625499</v>
       </c>
       <c r="AH42" s="33" t="n">
         <f aca="false">AH28-AH40</f>
-        <v>30242.1475040017</v>
+        <v>34812.8343481398</v>
       </c>
       <c r="AI42" s="33" t="n">
         <f aca="false">AI28-AI40</f>
-        <v>31779.1061304588</v>
+        <v>36309.8378084097</v>
       </c>
       <c r="AJ42" s="33" t="n">
         <f aca="false">AJ28-AJ40</f>
-        <v>33302.6292625499</v>
+        <v>37793.7550468321</v>
       </c>
       <c r="AK42" s="33" t="n">
         <f aca="false">AK28-AK40</f>
-        <v>34812.8343481398</v>
+        <v>39264.7004580672</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8910,135 +8910,135 @@
       </c>
       <c r="E44" s="17" t="n">
         <f aca="false">E42-E43</f>
-        <v>-2658.33333333333</v>
+        <v>-783.383333333333</v>
       </c>
       <c r="F44" s="17" t="n">
         <f aca="false">F42-F43</f>
-        <v>-2658.33333333333</v>
+        <v>-552.089709222762</v>
       </c>
       <c r="G44" s="17" t="n">
         <f aca="false">G42-G43</f>
-        <v>-2658.33333333333</v>
+        <v>-322.817963990467</v>
       </c>
       <c r="H44" s="17" t="n">
         <f aca="false">H42-H43</f>
-        <v>-783.383333333333</v>
+        <v>3479.23291017543</v>
       </c>
       <c r="I44" s="17" t="n">
         <f aca="false">I42-I43</f>
-        <v>-552.089709222762</v>
+        <v>4101.01712220154</v>
       </c>
       <c r="J44" s="17" t="n">
         <f aca="false">J42-J43</f>
-        <v>-322.817963990467</v>
+        <v>4717.36593854833</v>
       </c>
       <c r="K44" s="17" t="n">
         <f aca="false">K42-K43</f>
-        <v>3479.23291017543</v>
+        <v>1753.5435399969</v>
       </c>
       <c r="L44" s="17" t="n">
         <f aca="false">L42-L43</f>
-        <v>4101.01712220154</v>
+        <v>1962.66033636031</v>
       </c>
       <c r="M44" s="17" t="n">
         <f aca="false">M42-M43</f>
-        <v>4717.36593854833</v>
+        <v>2169.94911504581</v>
       </c>
       <c r="N44" s="17" t="n">
         <f aca="false">N42-N43</f>
-        <v>3769.91929321593</v>
+        <v>11175.4163903236</v>
       </c>
       <c r="O44" s="17" t="n">
         <f aca="false">O42-O43</f>
-        <v>4203.39657383107</v>
+        <v>12886.2607913919</v>
       </c>
       <c r="P44" s="17" t="n">
         <f aca="false">P42-P43</f>
-        <v>4633.08456470137</v>
+        <v>14582.149656302</v>
       </c>
       <c r="Q44" s="17" t="n">
         <f aca="false">Q42-Q43</f>
-        <v>11175.4163903236</v>
+        <v>10146.8137205327</v>
       </c>
       <c r="R44" s="17" t="n">
         <f aca="false">R42-R43</f>
-        <v>12886.2607913919</v>
+        <v>10524.5466709651</v>
       </c>
       <c r="S44" s="17" t="n">
         <f aca="false">S42-S43</f>
-        <v>14582.149656302</v>
+        <v>10898.9776269</v>
       </c>
       <c r="T44" s="17" t="n">
         <f aca="false">T42-T43</f>
-        <v>10146.8137205327</v>
+        <v>17386.5354530887</v>
       </c>
       <c r="U44" s="17" t="n">
         <f aca="false">U42-U43</f>
-        <v>10524.5466709651</v>
+        <v>19043.084667717</v>
       </c>
       <c r="V44" s="17" t="n">
         <f aca="false">V42-V43</f>
-        <v>10898.9776269</v>
+        <v>20685.1529735837</v>
       </c>
       <c r="W44" s="17" t="n">
         <f aca="false">W42-W43</f>
-        <v>17386.5354530887</v>
+        <v>22312.8669571595</v>
       </c>
       <c r="X44" s="17" t="n">
         <f aca="false">X42-X43</f>
-        <v>19043.084667717</v>
+        <v>23926.3520983453</v>
       </c>
       <c r="Y44" s="17" t="n">
         <f aca="false">Y42-Y43</f>
-        <v>20685.1529735837</v>
+        <v>25525.7327801458</v>
       </c>
       <c r="Z44" s="17" t="n">
         <f aca="false">Z42-Z43</f>
-        <v>21487.8669571595</v>
+        <v>20169.7322982574</v>
       </c>
       <c r="AA44" s="17" t="n">
         <f aca="false">AA42-AA43</f>
-        <v>23101.3520983453</v>
+        <v>20452.6369648151</v>
       </c>
       <c r="AB44" s="17" t="n">
         <f aca="false">AB42-AB43</f>
-        <v>24700.7327801458</v>
+        <v>20733.0685888404</v>
       </c>
       <c r="AC44" s="17" t="n">
         <f aca="false">AC42-AC43</f>
-        <v>20169.7322982574</v>
+        <v>27127.4487887092</v>
       </c>
       <c r="AD44" s="17" t="n">
         <f aca="false">AD42-AD43</f>
-        <v>20452.6369648151</v>
+        <v>28691.6348995764</v>
       </c>
       <c r="AE44" s="17" t="n">
         <f aca="false">AE42-AE43</f>
-        <v>20733.0685888404</v>
+        <v>30242.1475040017</v>
       </c>
       <c r="AF44" s="17" t="n">
         <f aca="false">AF42-AF43</f>
-        <v>27127.4487887092</v>
+        <v>31779.1061304588</v>
       </c>
       <c r="AG44" s="17" t="n">
         <f aca="false">AG42-AG43</f>
-        <v>28691.6348995764</v>
+        <v>33302.6292625499</v>
       </c>
       <c r="AH44" s="17" t="n">
         <f aca="false">AH42-AH43</f>
-        <v>30242.1475040017</v>
+        <v>34812.8343481398</v>
       </c>
       <c r="AI44" s="17" t="n">
         <f aca="false">AI42-AI43</f>
-        <v>31779.1061304588</v>
+        <v>36309.8378084097</v>
       </c>
       <c r="AJ44" s="17" t="n">
         <f aca="false">AJ42-AJ43</f>
-        <v>33302.6292625499</v>
+        <v>37793.7550468321</v>
       </c>
       <c r="AK44" s="17" t="n">
         <f aca="false">AK42-AK43</f>
-        <v>34812.8343481398</v>
+        <v>39264.7004580672</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9059,135 +9059,135 @@
       </c>
       <c r="E45" s="33" t="n">
         <f aca="false">D45+E44</f>
-        <v>-16133.3333333333</v>
+        <v>-14258.3833333333</v>
       </c>
       <c r="F45" s="33" t="n">
         <f aca="false">E45+F44</f>
-        <v>-18791.6666666667</v>
+        <v>-14810.4730425561</v>
       </c>
       <c r="G45" s="33" t="n">
         <f aca="false">F45+G44</f>
-        <v>-21450</v>
+        <v>-15133.2910065466</v>
       </c>
       <c r="H45" s="33" t="n">
         <f aca="false">G45+H44</f>
-        <v>-22233.3833333333</v>
+        <v>-11654.0580963711</v>
       </c>
       <c r="I45" s="33" t="n">
         <f aca="false">H45+I44</f>
-        <v>-22785.4730425561</v>
+        <v>-7553.04097416959</v>
       </c>
       <c r="J45" s="33" t="n">
         <f aca="false">I45+J44</f>
-        <v>-23108.2910065466</v>
+        <v>-2835.67503562126</v>
       </c>
       <c r="K45" s="33" t="n">
         <f aca="false">J45+K44</f>
-        <v>-19629.0580963711</v>
+        <v>-1082.13149562436</v>
       </c>
       <c r="L45" s="33" t="n">
         <f aca="false">K45+L44</f>
-        <v>-15528.0409741696</v>
+        <v>880.528840735952</v>
       </c>
       <c r="M45" s="33" t="n">
         <f aca="false">L45+M44</f>
-        <v>-10810.6750356213</v>
+        <v>3050.47795578176</v>
       </c>
       <c r="N45" s="33" t="n">
         <f aca="false">M45+N44</f>
-        <v>-7040.75574240533</v>
+        <v>14225.8943461053</v>
       </c>
       <c r="O45" s="33" t="n">
         <f aca="false">N45+O44</f>
-        <v>-2837.35916857426</v>
+        <v>27112.1551374972</v>
       </c>
       <c r="P45" s="33" t="n">
         <f aca="false">O45+P44</f>
-        <v>1795.72539612711</v>
+        <v>41694.3047937992</v>
       </c>
       <c r="Q45" s="33" t="n">
         <f aca="false">P45+Q44</f>
-        <v>12971.1417864507</v>
+        <v>51841.1185143319</v>
       </c>
       <c r="R45" s="33" t="n">
         <f aca="false">Q45+R44</f>
-        <v>25857.4025778426</v>
+        <v>62365.665185297</v>
       </c>
       <c r="S45" s="33" t="n">
         <f aca="false">R45+S44</f>
-        <v>40439.5522341446</v>
+        <v>73264.6428121969</v>
       </c>
       <c r="T45" s="33" t="n">
         <f aca="false">S45+T44</f>
-        <v>50586.3659546773</v>
+        <v>90651.1782652856</v>
       </c>
       <c r="U45" s="33" t="n">
         <f aca="false">T45+U44</f>
-        <v>61110.9126256423</v>
+        <v>109694.262933003</v>
       </c>
       <c r="V45" s="33" t="n">
         <f aca="false">U45+V44</f>
-        <v>72009.8902525423</v>
+        <v>130379.415906586</v>
       </c>
       <c r="W45" s="33" t="n">
         <f aca="false">V45+W44</f>
-        <v>89396.425705631</v>
+        <v>152692.282863746</v>
       </c>
       <c r="X45" s="33" t="n">
         <f aca="false">W45+X44</f>
-        <v>108439.510373348</v>
+        <v>176618.634962091</v>
       </c>
       <c r="Y45" s="33" t="n">
         <f aca="false">X45+Y44</f>
-        <v>129124.663346932</v>
+        <v>202144.367742237</v>
       </c>
       <c r="Z45" s="33" t="n">
         <f aca="false">Y45+Z44</f>
-        <v>150612.530304091</v>
+        <v>222314.100040494</v>
       </c>
       <c r="AA45" s="33" t="n">
         <f aca="false">Z45+AA44</f>
-        <v>173713.882402437</v>
+        <v>242766.737005309</v>
       </c>
       <c r="AB45" s="33" t="n">
         <f aca="false">AA45+AB44</f>
-        <v>198414.615182582</v>
+        <v>263499.80559415</v>
       </c>
       <c r="AC45" s="33" t="n">
         <f aca="false">AB45+AC44</f>
-        <v>218584.34748084</v>
+        <v>290627.254382859</v>
       </c>
       <c r="AD45" s="33" t="n">
         <f aca="false">AC45+AD44</f>
-        <v>239036.984445655</v>
+        <v>319318.889282435</v>
       </c>
       <c r="AE45" s="33" t="n">
         <f aca="false">AD45+AE44</f>
-        <v>259770.053034495</v>
+        <v>349561.036786437</v>
       </c>
       <c r="AF45" s="33" t="n">
         <f aca="false">AE45+AF44</f>
-        <v>286897.501823204</v>
+        <v>381340.142916896</v>
       </c>
       <c r="AG45" s="33" t="n">
         <f aca="false">AF45+AG44</f>
-        <v>315589.136722781</v>
+        <v>414642.772179446</v>
       </c>
       <c r="AH45" s="33" t="n">
         <f aca="false">AG45+AH44</f>
-        <v>345831.284226782</v>
+        <v>449455.606527586</v>
       </c>
       <c r="AI45" s="33" t="n">
         <f aca="false">AH45+AI44</f>
-        <v>377610.390357241</v>
+        <v>485765.444335995</v>
       </c>
       <c r="AJ45" s="33" t="n">
         <f aca="false">AI45+AJ44</f>
-        <v>410913.019619791</v>
+        <v>523559.199382827</v>
       </c>
       <c r="AK45" s="33" t="n">
         <f aca="false">AJ45+AK44</f>
-        <v>445725.853967931</v>
+        <v>562823.899840895</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9208,135 +9208,135 @@
       </c>
       <c r="E47" s="17" t="n">
         <f aca="false">(E12*Assumptions!$B$12+E13*Assumptions!$C$12+E14*Assumptions!$D$12)*12*(1-Assumptions!$B$31*Assumptions!$B$32)</f>
-        <v>0</v>
+        <v>6000</v>
       </c>
       <c r="F47" s="17" t="n">
         <f aca="false">(F12*Assumptions!$B$12+F13*Assumptions!$C$12+F14*Assumptions!$D$12)*12*(1-Assumptions!$B$31*Assumptions!$B$32)</f>
-        <v>0</v>
+        <v>11947.5503342718</v>
       </c>
       <c r="G47" s="17" t="n">
         <f aca="false">(G12*Assumptions!$B$12+G13*Assumptions!$C$12+G14*Assumptions!$D$12)*12*(1-Assumptions!$B$31*Assumptions!$B$32)</f>
-        <v>0</v>
+        <v>17843.109497388</v>
       </c>
       <c r="H47" s="17" t="n">
         <f aca="false">(H12*Assumptions!$B$12+H13*Assumptions!$C$12+H14*Assumptions!$D$12)*12*(1-Assumptions!$B$31*Assumptions!$B$32)</f>
-        <v>6000</v>
+        <v>33687.1319759397</v>
       </c>
       <c r="I47" s="17" t="n">
         <f aca="false">(I12*Assumptions!$B$12+I13*Assumptions!$C$12+I14*Assumptions!$D$12)*12*(1-Assumptions!$B$31*Assumptions!$B$32)</f>
-        <v>11947.5503342718</v>
+        <v>49392.6521740266</v>
       </c>
       <c r="J47" s="17" t="n">
         <f aca="false">(J12*Assumptions!$B$12+J13*Assumptions!$C$12+J14*Assumptions!$D$12)*12*(1-Assumptions!$B$31*Assumptions!$B$32)</f>
-        <v>17843.109497388</v>
+        <v>64960.8808247006</v>
       </c>
       <c r="K47" s="17" t="n">
         <f aca="false">(K12*Assumptions!$B$12+K13*Assumptions!$C$12+K14*Assumptions!$D$12)*12*(1-Assumptions!$B$31*Assumptions!$B$32)</f>
-        <v>33687.1319759397</v>
+        <v>70393.0180772566</v>
       </c>
       <c r="L47" s="17" t="n">
         <f aca="false">(L12*Assumptions!$B$12+L13*Assumptions!$C$12+L14*Assumptions!$D$12)*12*(1-Assumptions!$B$31*Assumptions!$B$32)</f>
-        <v>49392.6521740266</v>
+        <v>75777.6696992983</v>
       </c>
       <c r="M47" s="17" t="n">
         <f aca="false">(M12*Assumptions!$B$12+M13*Assumptions!$C$12+M14*Assumptions!$D$12)*12*(1-Assumptions!$B$31*Assumptions!$B$32)</f>
-        <v>64960.8808247006</v>
+        <v>81115.2507917335</v>
       </c>
       <c r="N47" s="17" t="n">
         <f aca="false">(N12*Assumptions!$B$12+N13*Assumptions!$C$12+N14*Assumptions!$D$12)*12*(1-Assumptions!$B$31*Assumptions!$B$32)</f>
-        <v>70393.0180772566</v>
+        <v>102406.17282682</v>
       </c>
       <c r="O47" s="17" t="n">
         <f aca="false">(O12*Assumptions!$B$12+O13*Assumptions!$C$12+O14*Assumptions!$D$12)*12*(1-Assumptions!$B$31*Assumptions!$B$32)</f>
-        <v>75777.6696992983</v>
+        <v>123510.977904608</v>
       </c>
       <c r="P47" s="17" t="n">
         <f aca="false">(P12*Assumptions!$B$12+P13*Assumptions!$C$12+P14*Assumptions!$D$12)*12*(1-Assumptions!$B$31*Assumptions!$B$32)</f>
-        <v>81115.2507917335</v>
+        <v>144431.292987132</v>
       </c>
       <c r="Q47" s="17" t="n">
         <f aca="false">(Q12*Assumptions!$B$12+Q13*Assumptions!$C$12+Q14*Assumptions!$D$12)*12*(1-Assumptions!$B$31*Assumptions!$B$32)</f>
-        <v>102406.17282682</v>
+        <v>149168.730814155</v>
       </c>
       <c r="R47" s="17" t="n">
         <f aca="false">(R12*Assumptions!$B$12+R13*Assumptions!$C$12+R14*Assumptions!$D$12)*12*(1-Assumptions!$B$31*Assumptions!$B$32)</f>
-        <v>123510.977904608</v>
+        <v>153864.755802771</v>
       </c>
       <c r="S47" s="17" t="n">
         <f aca="false">(S12*Assumptions!$B$12+S13*Assumptions!$C$12+S14*Assumptions!$D$12)*12*(1-Assumptions!$B$31*Assumptions!$B$32)</f>
-        <v>144431.292987132</v>
+        <v>158519.729967904</v>
       </c>
       <c r="T47" s="17" t="n">
         <f aca="false">(T12*Assumptions!$B$12+T13*Assumptions!$C$12+T14*Assumptions!$D$12)*12*(1-Assumptions!$B$31*Assumptions!$B$32)</f>
-        <v>149168.730814155</v>
+        <v>179134.012159881</v>
       </c>
       <c r="U47" s="17" t="n">
         <f aca="false">(U12*Assumptions!$B$12+U13*Assumptions!$C$12+U14*Assumptions!$D$12)*12*(1-Assumptions!$B$31*Assumptions!$B$32)</f>
-        <v>153864.755802771</v>
+        <v>199568.092316826</v>
       </c>
       <c r="V47" s="17" t="n">
         <f aca="false">(V12*Assumptions!$B$12+V13*Assumptions!$C$12+V14*Assumptions!$D$12)*12*(1-Assumptions!$B$31*Assumptions!$B$32)</f>
-        <v>158519.729967904</v>
+        <v>219823.545694821</v>
       </c>
       <c r="W47" s="17" t="n">
         <f aca="false">(W12*Assumptions!$B$12+W13*Assumptions!$C$12+W14*Assumptions!$D$12)*12*(1-Assumptions!$B$31*Assumptions!$B$32)</f>
-        <v>179134.012159881</v>
+        <v>239901.933779675</v>
       </c>
       <c r="X47" s="17" t="n">
         <f aca="false">(X12*Assumptions!$B$12+X13*Assumptions!$C$12+X14*Assumptions!$D$12)*12*(1-Assumptions!$B$31*Assumptions!$B$32)</f>
-        <v>199568.092316826</v>
+        <v>259804.804407293</v>
       </c>
       <c r="Y47" s="17" t="n">
         <f aca="false">(Y12*Assumptions!$B$12+Y13*Assumptions!$C$12+Y14*Assumptions!$D$12)*12*(1-Assumptions!$B$31*Assumptions!$B$32)</f>
-        <v>219823.545694821</v>
+        <v>279533.691883004</v>
       </c>
       <c r="Z47" s="17" t="n">
         <f aca="false">(Z12*Assumptions!$B$12+Z13*Assumptions!$C$12+Z14*Assumptions!$D$12)*12*(1-Assumptions!$B$31*Assumptions!$B$32)</f>
-        <v>239901.933779675</v>
+        <v>283090.117099832</v>
       </c>
       <c r="AA47" s="17" t="n">
         <f aca="false">(AA12*Assumptions!$B$12+AA13*Assumptions!$C$12+AA14*Assumptions!$D$12)*12*(1-Assumptions!$B$31*Assumptions!$B$32)</f>
-        <v>259804.804407293</v>
+        <v>286615.453431026</v>
       </c>
       <c r="AB47" s="17" t="n">
         <f aca="false">(AB12*Assumptions!$B$12+AB13*Assumptions!$C$12+AB14*Assumptions!$D$12)*12*(1-Assumptions!$B$31*Assumptions!$B$32)</f>
-        <v>279533.691883004</v>
+        <v>290109.972643528</v>
       </c>
       <c r="AC47" s="17" t="n">
         <f aca="false">(AC12*Assumptions!$B$12+AC13*Assumptions!$C$12+AC14*Assumptions!$D$12)*12*(1-Assumptions!$B$31*Assumptions!$B$32)</f>
-        <v>283090.117099832</v>
+        <v>309573.944128601</v>
       </c>
       <c r="AD47" s="17" t="n">
         <f aca="false">(AD12*Assumptions!$B$12+AD13*Assumptions!$C$12+AD14*Assumptions!$D$12)*12*(1-Assumptions!$B$31*Assumptions!$B$32)</f>
-        <v>286615.453431026</v>
+        <v>328867.769147317</v>
       </c>
       <c r="AE47" s="17" t="n">
         <f aca="false">(AE12*Assumptions!$B$12+AE13*Assumptions!$C$12+AE14*Assumptions!$D$12)*12*(1-Assumptions!$B$31*Assumptions!$B$32)</f>
-        <v>290109.972643528</v>
+        <v>347992.935053893</v>
       </c>
       <c r="AF47" s="17" t="n">
         <f aca="false">(AF12*Assumptions!$B$12+AF13*Assumptions!$C$12+AF14*Assumptions!$D$12)*12*(1-Assumptions!$B$31*Assumptions!$B$32)</f>
-        <v>309573.944128601</v>
+        <v>366950.916200668</v>
       </c>
       <c r="AG47" s="17" t="n">
         <f aca="false">(AG12*Assumptions!$B$12+AG13*Assumptions!$C$12+AG14*Assumptions!$D$12)*12*(1-Assumptions!$B$31*Assumptions!$B$32)</f>
-        <v>328867.769147317</v>
+        <v>385743.174051773</v>
       </c>
       <c r="AH47" s="17" t="n">
         <f aca="false">(AH12*Assumptions!$B$12+AH13*Assumptions!$C$12+AH14*Assumptions!$D$12)*12*(1-Assumptions!$B$31*Assumptions!$B$32)</f>
-        <v>347992.935053893</v>
+        <v>404371.157295782</v>
       </c>
       <c r="AI47" s="17" t="n">
         <f aca="false">(AI12*Assumptions!$B$12+AI13*Assumptions!$C$12+AI14*Assumptions!$D$12)*12*(1-Assumptions!$B$31*Assumptions!$B$32)</f>
-        <v>366950.916200668</v>
+        <v>422836.301957402</v>
       </c>
       <c r="AJ47" s="17" t="n">
         <f aca="false">(AJ12*Assumptions!$B$12+AJ13*Assumptions!$C$12+AJ14*Assumptions!$D$12)*12*(1-Assumptions!$B$31*Assumptions!$B$32)</f>
-        <v>385743.174051773</v>
+        <v>441140.031508168</v>
       </c>
       <c r="AK47" s="17" t="n">
         <f aca="false">(AK12*Assumptions!$B$12+AK13*Assumptions!$C$12+AK14*Assumptions!$D$12)*12*(1-Assumptions!$B$31*Assumptions!$B$32)</f>
-        <v>404371.157295782</v>
+        <v>459283.756976181</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9369,15 +9369,15 @@
       </c>
       <c r="H48" s="20" t="n">
         <f aca="false">IF(AND(H42&gt;=0,I48&lt;&gt;999),H$2,999)</f>
-        <v>999</v>
+        <v>7</v>
       </c>
       <c r="I48" s="20" t="n">
         <f aca="false">IF(AND(I42&gt;=0,J48&lt;&gt;999),I$2,999)</f>
-        <v>999</v>
+        <v>8</v>
       </c>
       <c r="J48" s="20" t="n">
         <f aca="false">IF(AND(J42&gt;=0,K48&lt;&gt;999),J$2,999)</f>
-        <v>999</v>
+        <v>9</v>
       </c>
       <c r="K48" s="20" t="n">
         <f aca="false">IF(AND(K42&gt;=0,L48&lt;&gt;999),K$2,999)</f>

</xml_diff>